<commit_message>
Alune's page (docs/heroes/tft_alune.md: the dev record - kit picks, balance, add-on, sprite, effects, sounds, card) and the README table (175 heroes, tft 2); gen_hero_docs says a tft add-on installs on its own (not in league_addons); CI checks tft_alune's copy and runs its tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11537,63 +11537,128 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
+          <t>拉露恩</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Alune</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>tft_alune</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>中单</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
+（攻击间隔 1.5 秒 · 攻击距离 55000）</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>月之降临：月光碎片从天而降，落在3个敌人身上（一个是目标），每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
+（冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
+（冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：范围内的敌人受到165 + 72% 法强魔法伤害，中心的敌人眩晕0.83秒。
+（冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>拉露恩附加包（tft_alune v0.1.0）
+月之降临：落在离她最近的 q_n 个敌人身上（金铲铲的规则），每枚 q_dmg + q_ratio% 法强、月蚀印记（魔抗 -q_shred%）
+月曜降临：整颗月亮的伤害（含月相加成）× r_split% 由命中的敌人平分，每人最多 r_cap%：只砸中一个人时最痛
+普攻：月环飞回来，穿过路上的每个敌人（a_back_r% 攻击力），打中的那个人回来时再挨一下</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C176" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E175" s="2" t="inlineStr">
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G175" s="2" t="inlineStr">
+      <c r="G176" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H175" s="2" t="inlineStr">
+      <c r="H176" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="inlineStr">
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
-      <c r="L175" s="3" t="inlineStr">
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L175"/>
+  <autoFilter ref="A1:L176"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -11769,6 +11834,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId175"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Vayne PPU 2.2 registered (「通过，继续注册薇恩」): league.dll 0.7.172 (hd.rs row, drawn at 2.55, no SIZES row: 40 game px as before), main 0.235.0; Illaoi's spirit (only league_vayne/_l) and Viego's souls (her hd_/lo_ tags); preview_vayne on the dense frames; hero page, gallery, tech notes (and the hero pages main left with old add-on versions)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -4207,7 +4207,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.1）
+          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.2）
 易：每一次英雄击杀和助攻，阿尔法突袭和冥想的剩余冷却减 70%，无极剑道开着时再延长 4 秒；每次普攻阿尔法突袭冷却减 1 秒；无极剑道期间免疫减速</t>
         </is>
       </c>
@@ -5998,7 +5998,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>阿兹尔附加包（league_azir v0.1.2）
+          <t>阿兹尔附加包（league_azir v0.1.3）
 太阳圆盘（并入被动，英雄联盟的「恕瑞玛的传承」）：开局记下我方每座塔；每局一次，某座塔倒了、阿兹尔走到废墟 d_near（60000）内、废墟 d_range（45000）内有敌人时，圆盘从沙里升起，立 d_life tick（…
 禁军之墙的禁军：按阿兹尔到大招目标的方向朝左或朝右（反推时他已经绕到目标身后，禁军就朝回冲）；伤害和击退还是数据那道墙的
 沙兵（用户：「沙兵没攻击动作 你想办法补吧 不让codex了 还有不面向敌人」）：从侧面画：升起，之后每 ss_stand tick（4）盖一次站姿，朝 60 像素内最近的敌人（先英雄，敌人正好在它上下方时不转）；刺过以后下一次改放刺击（ss_stab tic…</t>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.8）
+          <t>塞拉斯附加包（league_sylas v0.2.9）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>塔莉垭附加包（league_taliyah v0.1.0）
+          <t>塔莉垭附加包（league_taliyah v0.2.0）
 竖墙（敌人近、或她已在打架）：同一块地方是真的墙：英雄、小兵、野怪、召唤物（两边都算，她自己也算）都过不去；立起时压在上面的单位推到她那一侧
 横墙（敌人远：骑墙）：每一段都是真的墙；她骑墙时站在墙顶上不受挡，跳下来那一 tick 推到近的一侧</t>
         </is>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.1）
+          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.2）
 金克丝：每一次英雄击杀和助攻（几个人同时阵亡也各算一次）</t>
         </is>
       </c>
@@ -8863,7 +8863,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>卡莉丝塔附加包（league_kalista v0.1.1）
+          <t>卡莉丝塔附加包（league_kalista v0.1.2）
 武术姿态：每次投矛后自己判断往前还是往后：最近的敌方英雄残血（40% 以下），或者它在逃（越跑越远）而且快跑出射程（超过攻击距离 80%），就往前追；其余都往后跳开；身边没有敌方英雄时照主…
 誓约者：开局绑定一名队友（辅助位优先，没有就最近的队友英雄，每条命出生时重新看），大招对誓约者施放
 命运的召唤：把誓约者拉进来保护、定身，然后逐 tick 飞向离她最近的敌方英雄现在的位置（90000 内，没有就两倍范围），到了就在脚下击飞周围敌人
@@ -9439,7 +9439,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.1）
+          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.2）
 崔丝塔娜：每一次英雄击杀和助攻都刷新（满层引爆照旧）</t>
         </is>
       </c>
@@ -9502,7 +9502,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.1）
+          <t>参与击杀附加包：金克丝、崔丝塔娜、易、图奇（league_takedowns v0.3.2）
 图奇：埋伏助攻也刷新；E 等到有人满 6 层毒、或这一爆能毒死人才引爆（v0.3.0），条件一满足下一箭就爆（v0.3.1）</t>
         </is>
       </c>
@@ -9637,7 +9637,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Lucian PPU 2.02 registered (「通过，继续注册卢锡安」): league.dll 0.7.173 (hd.rs row, no SIZES row: 46 game px as before), main 0.236.0; Illaoi's spirit (only league_lucian/_l) and Viego's souls (his hd_/lo_ tags); preview_lucian on the dense frames, Nami's, Ryze's, Sona's and Zilean's showcases with the new him; hero page, gallery, tech notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>青钢影钩墙附加包（league_camille_wall v0.4.4）
+          <t>青钢影钩墙附加包（league_camille_wall v0.4.5）
 主包 league 保持纯数据、全平台可用；钩墙要读地图的墙，只能用原生代码，所以放在这个单独的附加包里。 装上后，青钢影的 E「钩索」钩墙、地图四边和防御塔，不再钩小兵、野怪；英雄、树林、草丛也不钩（墙就在树林里）。
 游戏 AI 不按的技能替它按（league_ult_press v0.5.5）
 卡蜜尔 E：E 好了、60000 内有敌方英雄就按，目标是最近的那个（钩墙附加包的 E 射程是 85000，取小的）。钩索、钩墙、冲向敌人照旧由主包 / 钩墙附加包决定</t>
@@ -750,13 +750,13 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>盛宴：吞噬受伤的敌方英雄，造成300 + 自身5%最大生命的真实伤害和50% 法强无视魔抗的魔法伤害；吃掉则叠一层：最大生命+70、体型变大（不封顶，死亡清空）。
+          <t>盛宴：吞噬受伤的敌方英雄，造成300 + 自身5%最大生命的真实伤害和50% 法强无视魔抗的魔法伤害；吃掉则叠一层：最大生命+70、体型变大（最多 2 倍，死亡清空）。
 （冷却 60 秒 · 施放距离 30000 · 施放：指定目标 · 刚交过手的敌方英雄）</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>科加斯附加包（league_chogath v0.1.0）
+          <t>科加斯附加包（league_chogath v0.1.1）
 盛宴的层数：死后原样补回，层数一局里只增不减
 什么时候放盛宴：读射程内敌方英雄的生命、护盾、免死和受到伤害的增减，一口吃得死才放（几个时吃生命 + 护盾最少的，AI 没想放也放）；吃不死时 AI 想放就改成普攻那个人</t>
         </is>
@@ -8995,7 +8995,7 @@
       <c r="I134" s="2" t="inlineStr"/>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Silco: hero page, README table, docs regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$178</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.14）
+          <t>俄洛伊附加包（league_illaoi v0.2.15）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -4976,7 +4976,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>希瓦娜附加包（league_shyvana v0.1.0）
+          <t>希瓦娜附加包（league_shyvana v0.1.1）
 龙形的样子：整身变龙：龙形期间（league_shyvana_dg，和龙形刚结束、还没播变回动作时的 league_shyvana_was_dg）站、跑、挨打、阵亡都换成 d_idle / …</t>
         </is>
       </c>
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.3）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.4）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.9）
+          <t>塞拉斯附加包（league_sylas v0.2.10）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11708,8 +11708,66 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>希尔科</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Silco</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>tft_silco</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>中单</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
+（攻击间隔 1.5 秒 · 攻击距离 55000）</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
+（冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
+（冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
+（冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L177"/>
+  <autoFilter ref="A1:L178"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -11887,6 +11945,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId174"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId175"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId177"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Maddie: hero page, README table, docs regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L178"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.15）
+          <t>俄洛伊附加包（league_illaoi v0.2.16）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.4）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.5）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.10）
+          <t>塞拉斯附加包（league_sylas v0.2.11）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11766,8 +11766,66 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>麦迪</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Maddie</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>tft_maddie</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>ADC</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
+（攻击间隔 1.1 秒 · 攻击距离 68000）</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
+（冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
+（冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
+（冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L178"/>
+  <autoFilter ref="A1:L179"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -11946,6 +12004,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId175"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId178"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Loris: hero page, README table, docs regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$180</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.16）
+          <t>俄洛伊附加包（league_illaoi v0.2.17）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.5）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.6）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.11）
+          <t>塞拉斯附加包（league_sylas v0.2.12）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11824,8 +11824,66 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>洛里斯</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Loris</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>tft_loris</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>辅助</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
+（攻击间隔 1.4 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
+（冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
+（冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
+（冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L179"/>
+  <autoFilter ref="A1:L180"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12005,6 +12063,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId179"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Kobuko: Sylas steals Game Over! with its effects (46 events in the steal check), Viego/Neeko souls (melee), Illaoi's ghost (179), Kayn ranges; hero page, README table, docs; versions main 0.240.0 / league.dll 0.7.178 / illaoi 0.2.18 / sylas 0.2.13 / viego_soul 0.2.7 / tft 0.8.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.17）
+          <t>俄洛伊附加包（league_illaoi v0.2.18）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.6）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.7）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.12）
+          <t>塞拉斯附加包（league_sylas v0.2.13）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11537,353 +11537,411 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
+          <t>可酷伯</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Kobuko</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>tft_kobuko</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>猫爪掌，造成100% 攻击力物理伤害。第二阶段：每条命第一次生命低于50%时进入狂怒，直到阵亡：攻击速度+40%、生命偷取20%。
+（攻击间隔 1.2 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>金爪真言：获得70 + 50% 法强的护盾（4秒）；4秒内下一次普攻变为金爪重掌，造成40 + 105% 攻击力 + 2%最大生命物理伤害并晕眩1秒。
+（冷却 9.5 秒 · 施放距离 25000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>猛虎扑：扑向目标，落地时周围的敌人受到40 + 70% 攻击力 + 2%最大生命物理伤害并被击飞0.4秒。
+（冷却 10.5 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>游戏结束！：一跃冲天（期间不可选中、免疫控制），砸落在敌方英雄身上：目标受到70 + 100% 攻击力 + 6%最大生命物理伤害，周围的敌人（含目标）再受到70 + 60% 攻击力 + 3%最大生命物理伤害并被击飞0.8秒。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_kobuko.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C176" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E175" s="2" t="inlineStr">
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G175" s="2" t="inlineStr">
+      <c r="G176" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H175" s="2" t="inlineStr">
+      <c r="H176" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="inlineStr">
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
-      <c r="L175" s="3" t="inlineStr">
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L180"/>
+  <autoFilter ref="A1:L181"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12064,6 +12122,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId180"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Vander: hero page, README table, docs; Illaoi's ghost with Kobuko's (181); versions main 0.241.0 / league.dll 0.7.179 / illaoi 0.2.19 / sylas 0.2.14 / viego_soul 0.2.8 / tft 0.9.0 (Kobuko took 0.8.0); his reel tags back on the sheet (the run's re-export had dropped them)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.18）
+          <t>俄洛伊附加包（league_illaoi v0.2.19）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.7）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.8）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.13）
+          <t>塞拉斯附加包（league_sylas v0.2.14）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11595,353 +11595,411 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
+          <t>范德尔</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Vander</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>tft_vander</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
+（攻击间隔 1.07 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
+（冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L181"/>
+  <autoFilter ref="A1:L182"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12123,6 +12181,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId181"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Akali PPU 1.8 registered: league.dll 0.7.184 (hd.rs row), main 0.244.0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table); Sylas's copy regenerated (unchanged: he takes her R's effects, not her body); preview_akali on the dense frames; hero page, gallery, tech notes, README
40 game px as her 1x sprite: no SIZES row, the face point (1, -35) and the ban/pick value -10 stay (tfm2_ase face:
PASS, on her crown; bp_card_audit: -10 is the rule's). The kit's offsets stay (the same height and the old poses'
timing; the dashes baked as before).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5684,7 +5684,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr"/>
@@ -10556,7 +10556,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>冲击之潮：水流冲击敌人，造成65 + 45% 法术强度的魔法伤害，弹向附近友方英雄回复70 + 35% 法术强度的生命值，再弹向另一名敌方英雄造成60 + 40% 法术强度伤害。唤潮之佑：被治疗者4秒内攻击力和法术强度提高15%，被击中者减速25%。
+          <t>冲击之潮：水流先治疗身边一名友方英雄（没有则治疗自己）70 + 35% 法术强度的生命值，再弹向附近敌人造成65 + 45% 法术强度的魔法伤害，不会弹回娜美。唤潮之佑：被治疗者4秒内攻击力和法术强度提高15%，被击中者减速25%。
 （冷却 7 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>

</xml_diff>

<commit_message>
tft_violet: hero page, README table, previews; versions main 0.245.0 / league.dll 0.7.187 / illaoi 0.2.20 / sylas 0.2.15 / viego_soul 0.2.9 / tft 0.10.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$183</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L182"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -691,7 +691,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>青钢影钩墙附加包（league_camille_wall v0.4.5）
+          <t>青钢影钩墙附加包（league_camille_wall v0.4.6）
 主包 league 保持纯数据、全平台可用；钩墙要读地图的墙，只能用原生代码，所以放在这个单独的附加包里。 装上后，青钢影的 E「钩索」钩墙、地图四边和防御塔，不再钩小兵、野怪；英雄、树林、草丛也不钩（墙就在树林里）。
 游戏 AI 不按的技能替它按（league_ult_press v0.5.5）
 卡蜜尔 E：E 好了、60000 内有敌方英雄就按，目标是最近的那个（钩墙附加包的 E 射程是 85000，取小的）。钩索、钩墙、冲向敌人照旧由主包 / 钩墙附加包决定</t>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.19）
+          <t>俄洛伊附加包（league_illaoi v0.2.20）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.8）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.9）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.14）
+          <t>塞拉斯附加包（league_sylas v0.2.15）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -8992,10 +8992,15 @@
 （冷却 60 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I134" s="2" t="inlineStr"/>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>卢锡安附加包（league_lucian v0.1.0）
+Lucian walks firing The Culling (needs League of Legends Heroes): while his ult fires, his walk is drawn with both pistols levelled forward instead of his plain run. Picture only;…</t>
+        </is>
+      </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr"/>
@@ -11449,7 +11454,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.1）
+          <t>悠米附加包（league_yuumi v0.1.3）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11653,353 +11658,411 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
+          <t>蔚奥莱</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Violet</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>tft_violet</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
+（攻击间隔 0.93 秒 · 攻击距离 24000）</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
+（冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
+（冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L182"/>
+  <autoFilter ref="A1:L183"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12182,6 +12245,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId182"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ancient Krug: hero page, README table, previews; versions main 0.246.0 / league.dll 0.7.188 / illaoi 0.2.21 / sylas 0.2.16 / viego_soul 0.2.10 / yuumi 0.1.4 / tft 0.11.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$183</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$184</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L183"/>
+  <dimension ref="A1:L184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.20）
+          <t>俄洛伊附加包（league_illaoi v0.2.21）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.9）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.10）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.15）
+          <t>塞拉斯附加包（league_sylas v0.2.16）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11454,7 +11454,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.3）
+          <t>悠米附加包（league_yuumi v0.1.4）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11600,469 +11600,527 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
+          <t>远古石甲虫</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Krug</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>tft_krug</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
+（攻击间隔 1.2 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
+（冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L183"/>
+  <autoFilter ref="A1:L184"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12246,6 +12304,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId183"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ao Shin: hero page, README table, previews; versions main 0.247.0 / league.dll 0.7.189 / illaoi 0.2.22 / sylas 0.2.17 / viego_soul 0.2.11 / yuumi 0.1.5 / tft 0.13.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L184"/>
+  <dimension ref="A1:L185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.21）
+          <t>俄洛伊附加包（league_illaoi v0.2.22）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.10）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.11）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.16）
+          <t>塞拉斯附加包（league_sylas v0.2.17）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11454,7 +11454,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.4）
+          <t>悠米附加包（league_yuumi v0.1.5）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11832,295 +11832,353 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
+          <t>敖兴</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Ao Shin</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>tft_aoshin</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>中单</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
+（攻击间隔 1.5 秒 · 攻击距离 55000）</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
+（冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
+（冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
+（冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L184"/>
+  <autoFilter ref="A1:L185"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12305,6 +12363,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId184"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scar: hero page, README table, previews; versions main 0.248.0 / league.dll 0.7.190 / illaoi 0.2.23 / sylas 0.2.18 / viego_soul 0.2.12 / yuumi 0.1.6 / tft 0.14.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L185"/>
+  <dimension ref="A1:L186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.22）
+          <t>俄洛伊附加包（league_illaoi v0.2.23）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.11）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.12）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.17）
+          <t>塞拉斯附加包（league_sylas v0.2.18）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11454,7 +11454,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.5）
+          <t>悠米附加包（league_yuumi v0.1.6）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11600,585 +11600,643 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
+          <t>刀疤</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Scar</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>tft_scar</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>长矛刺击造成100% 攻击力物理伤害。野火冲刺：每6秒下一击踩滑板冲刺，造成40 + 110% 攻击力+30% 法强伤害，回复上次冲刺以来所受伤害的25%。监察：生命不低于50%时减伤20%，否则10%。
+（攻击间隔 1.2 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>水坑狙击惊喜：向最近的3名敌人各扔一颗炸弹，造成70 + 80% 法强魔法伤害并晕眩1秒；自己回复60 + 60% 法强生命。
+（冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>长矛横扫：长矛横扫前方，造成50 + 80% 攻击力+2% 最大生命物理伤害并击退敌人。
+（冷却 9 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>野火突袭：踩滑板冲向敌人，途中丢下两颗燃烧弹（各40 + 40% 法强魔法伤害）；落地爆炸，周围敌人受到120 + 100% 法强魔法伤害并被击飞0.5秒，之后4秒内减伤40%。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scar.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L185"/>
+  <autoFilter ref="A1:L186"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12364,6 +12422,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId185"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tristana PPU 2.56 registered: league.dll 0.7.192 (hd.rs row), main 0.250.0; idle_base held still; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table); Sylas's copy regenerated (unchanged); preview_tristana on the dense frames; hero page, gallery, tech notes, README
idle_base is now the design held still: her old idle sank a pixel in frames 3-5, but the bob is no longer played - the
idle is hero_reels' reel of action snippets (the user: 「现在不是随机动画吗 你还在上下晃动？」). 34 game px as her 1x
sprite: no SIZES row, the face point (-3, -28) stays (tfm2_ase face: PASS); her card needs no value (bp_card_audit: top
-23.3, no flag). The kit's offsets stay.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.12）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.13）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.18）
+          <t>塞拉斯附加包（league_sylas v0.2.19）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -9450,7 +9450,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="K141" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Zed PPU 1.62 registered: league.dll 0.7.193 (hd.rs row), main 0.251.0; Illaoi's spirit, Viego's souls (his hd_ / lo_ tags; Neeko reads the same table); preview_zed on the dense frames; hero page, gallery, tech notes, README
40 game px as his 1x sprite: no SIZES row, the face point (-1, -37) stays (tfm2_ase face: PASS); his card keeps -10
(bp_card_audit: the rule's -10, top -28.7). His shadow clones are their own effect pictures (league_zed_fx sh_*), as
tall as he is: unchanged. The idle and ban/pick reels are hero_reels' cuts of the new frames.

The game's latest update brought four base champions (bombardier, ferryman, gladiator, hypnotist): regenerated on it,
Sylas's class table and Viego's soul table (Neeko reads it) take them in - league_sylas 0.2.20, league_viego_soul
0.2.14 (their hero pages' version lines with them).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5292,7 +5292,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.13）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.14）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -6692,7 +6692,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.0）
+          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.1）
 乐芙兰 镜花水月：生命不高于 40%</t>
         </is>
       </c>
@@ -6755,7 +6755,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.0）
+          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.1）
 丽桑卓 大招冰封自己：生命不高于 35%</t>
         </is>
       </c>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.19）
+          <t>塞拉斯附加包（league_sylas v0.2.20）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -8043,7 +8043,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.0）
+          <t>低血量附加包：布里茨、乐芙兰、丽桑卓（league_lowhp v0.2.1）
 布里茨 法力屏障：生命不高于 30%</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Renni: hero page, README table, previews; versions main 0.253.0 / league.dll 0.8.1 / illaoi 0.2.24 / sylas 0.2.23 / viego_soul 0.2.16 / yuumi 0.1.7 / tft 0.15.0
The generated pages of Azir, Gangplank and Poppy caught up with their merged add-ons on the way.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$187</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L186"/>
+  <dimension ref="A1:L187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -691,7 +691,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>青钢影钩墙附加包（league_camille_wall v0.4.6）
+          <t>青钢影钩墙附加包（league_camille_wall v0.4.9）
 主包 league 保持纯数据、全平台可用；钩墙要读地图的墙，只能用原生代码，所以放在这个单独的附加包里。 装上后，青钢影的 E「钩索」钩墙、地图四边和防御塔，不再钩小兵、野怪；英雄、树林、草丛也不钩（墙就在树林里）。
 游戏 AI 不按的技能替它按（league_ult_press v0.5.5）
 卡蜜尔 E：E 好了、60000 内有敌方英雄就按，目标是最近的那个（钩墙附加包的 E 射程是 85000，取小的）。钩索、钩墙、冲向敌人照旧由主包 / 钩墙附加包决定</t>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>火药桶：向敌方英雄扔火药桶（最多2个，留8秒），1秒后引线点燃。被枪火谈判、贴身攻击或另一个桶的爆炸引爆：范围内敌人受到40 + 100% 攻击力物理伤害（英雄再加60），无视40%护甲，减速40%2秒。
+          <t>火药桶：向敌方英雄扔火药桶（最多3个，留8秒），1秒后引线点燃。被枪火谈判、贴身攻击或另一个桶的爆炸引爆：范围内敌人受到40 + 100% 攻击力物理伤害（英雄再加60），无视40%护甲，减速40%2秒。
 （冷却 8 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
@@ -1017,9 +1017,11 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>普朗克附加包（league_gangplank v0.1.0）
+          <t>普朗克附加包（league_gangplank v0.2.0）
 坏血病疗法（W）：同上，另外吃下去的那个 tick 清掉他身上的硬控（英雄联盟：W 解除控制）；生命低于 40% 也会吃
-火药桶连锁（E）：两个桶相距不超过 e_chain（70000）才连锁；桶边有敌人照样由数据炸，桶边没人也空炸（画面、声音、刷新烈火审讯和加速都有）</t>
+火药桶连锁（E）：两个桶相距不超过 e_chain（70000）才连锁；桶边有敌人照样由数据炸，桶边没人也空炸（画面、声音、刷新烈火审讯和加速都有），空炸的桶接着往下连
+火药桶充能（E）：能存 3 个桶（e_stock），每过一轮 E 的冷却回一个；手里还有桶时扔完只等 e_gap（60 tick）就能再扔
+三连桶（E + Q）：枪火谈判打中时，两个点燃的桶连着、有敌方英雄在其中一个桶的 e_chain 以内却不在任何桶的爆炸范围里、手里还有桶：往他脚下补第三个桶，离他最近的桶先炸，连锁带上另一个，6 t…</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1275,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.23）
+          <t>俄洛伊附加包（league_illaoi v0.2.24）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -3888,7 +3890,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>凯隐「暗裔魔镰」附加包（league_kayn_form v0.3.3）
+          <t>凯隐「暗裔魔镰」附加包（league_kayn_form v0.3.5）
 攒哪种形态：打中近战英雄攒暗裔、打中远程英雄攒影流（普攻和技能都算，各 14 次），按英雄的攻击距离分
 形态能留多久：整局：阵亡复活后光环和形态效果直接回来
 变身后的样子：整个身体都是形态的（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -4081,7 +4083,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>盲僧 W 位移附加包（league_leesin_hop v0.1.9）
+          <t>盲僧 W 位移附加包（league_leesin_hop v0.1.10）
 主包 league 保持纯数据。主包的李青不能「摸眼」：R 身后没人时直接冲过目标落到他身后回旋踢，W 并进了 E、不冲刺。 英雄联盟手游里李青的 W 不用插眼就能冲到一个点，这个附加包照这个做（不画眼）： - 回旋踢（照高手的打法，v0.1.6）：R 时目标身后没有别的敌方英雄（有人就照旧正面踢进人堆），第 7 tick 先定往哪踢—— 踢回自己队伍那边…</t>
         </is>
       </c>
@@ -4144,7 +4146,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>莉莉娅梦尘与昏睡附加包（league_lillia v0.1.2）
+          <t>莉莉娅梦尘与昏睡附加包（league_lillia v0.1.3）
 主包 league 保持纯数据。数据里能读最大生命值的只有真实伤害，也没有「受到伤害就醒」的效果，所以主包莉莉娅： 被动「梦满枝」的梦尘对英雄每 0.75 秒造成 1% 最大生命值的真实伤害；大招「夜阑谣」让带梦尘的敌方英雄困倦 1.5 秒后 眩晕 1.5 秒（打不醒），她的 Q / W 打到眩晕中的英雄时多造成一段惊醒伤害。英雄联盟里梦尘是魔法伤害，昏睡…</t>
         </is>
       </c>
@@ -5292,7 +5294,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.14）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.16）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -5998,7 +6000,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>阿兹尔附加包（league_azir v0.1.3）
+          <t>阿兹尔附加包（league_azir v0.1.4）
 太阳圆盘（并入被动，英雄联盟的「恕瑞玛的传承」）：开局记下我方每座塔；每局一次，某座塔倒了、阿兹尔走到废墟 d_near（60000）内、废墟 d_range（45000）内有敌人时，圆盘从沙里升起，立 d_life tick（…
 禁军之墙的禁军：按阿兹尔到大招目标的方向朝左或朝右（反推时他已经绕到目标身后，禁军就朝回冲）；伤害和击退还是数据那道墙的
 沙兵（用户：「沙兵没攻击动作 你想办法补吧 不让codex了 还有不面向敌人」）：从侧面画：升起，之后每 ss_stand tick（4）盖一次站姿，朝 60 像素内最近的敌人（先英雄，敌人正好在它上下方时不转）；刺过以后下一次改放刺击（ss_stab tic…</t>
@@ -7272,7 +7274,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.20）
+          <t>塞拉斯附加包（league_sylas v0.2.23）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -7464,7 +7466,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>泰隆「刺客之道」翻墙附加包（league_talon_vault v0.1.2）
+          <t>泰隆「刺客之道」翻墙附加包（league_talon_vault v0.1.3）
 什么时候翻：照旧，另外：残血（低于 35%）而身边有敌方英雄，或被围（身边敌方英雄 ≥ 2、比身边友方多、生命低于 70%）时；残血敌方英雄（≤ 60%）躲在墙后、他自己生命 ≥ 40% 时
 往哪翻：翻过墙：撤离时找背向敌人、16000 内的墙翻到另一边（落地后离敌人最远的那处）；追击时朝目标左右 35° 内找墙翻过去，落点要近 15000 以上、不翻进人堆
 冷却：同一个冷却（主包的 league_talon_e_cd），两种翻越不会连着出</t>
@@ -8152,7 +8154,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>催眠气泡：踢出气泡，打中敌方英雄造成60 + 40% 法强魔法伤害，困倦（减速30%）1.4秒后昏睡2秒；没打中就留在原地。昏睡中第一次被飞星打中伤害翻倍。
+          <t>催眠气泡：踢出气泡，打中敌方英雄造成60 + 40% 法强魔法伤害，困倦（减速30%）1.4秒后睡眠2秒，受到任何伤害就醒，打醒的那一下伤害提高100%；没打中就留在原地。
 （冷却 15 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
@@ -8164,8 +8166,8 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>佐伊附加包（league_zoe v0.3.0）
-催眠气泡的昏睡：照英雄联盟：困倦后昏睡 2.25 秒，受到任何伤害就醒（谁打的都算），那一下再来一遍真实伤害，最多 100 + 60% 法强
+          <t>佐伊附加包（league_zoe v0.4.0）
+催眠气泡的睡眠：一样是官方睡眠，2.25 秒（英雄联盟的时长）；睡着时头上有睡泡，醒了就摘掉，被打醒的放醒来的画面
 飞星的伤害：按真实飞行距离：出手点 20000 以内 100%，到 85000 线性加到 250%
 窃法巧手：另外：敌方英雄放大招时原地掉下一块法术碎片（20 秒，最多 3 块），她走到 18000 以内就捡起来，射 3 颗飞弹（打 70000 内最近的敌方英雄，每颗 45 + 15% …
 召唤师技能（0.2.0）：用户：「可以改成召唤师技能那种效果吗 随机的」「能做成智能释放吗」：窃法巧手每次发动（大招射飞弹的那一刻、捡起碎片时）先放一个召唤师技能，按局面挑：被控 → 净化；残血、敌方英雄…</t>
@@ -9379,7 +9381,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>斯莫德附加包（league_smolder v0.1.1）
+          <t>斯莫德附加包（league_smolder v0.1.2）
 龙之研习的层数：死后保留（层数、计数器、三档全部原样补回）
 三档龙息：灼烧之外，被打中的单位生命不高于最大生命的 6.5% 就处决（真实伤害，击杀算他的）
 扑棱，扑棱，扑棱！：自己的冷却（20 秒），好了就每 3 tick 看一次：撤——生命低于 40% 而 40000 内有敌方英雄、30000 内有敌方英雄、或 40000 内敌方英雄 2 名以上且比…</t>
@@ -9950,7 +9952,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>巴德「神奇旅程」穿墙门附加包（league_bard v0.6.1）
+          <t>巴德「神奇旅程」穿墙门附加包（league_bard v0.6.2）
 什么时候开门：冷却（16 秒）一好就每 3 tick 看一次：撤——生命低于 45% 而 30000 内有敌方英雄、15000 内有敌方英雄、或 30000 内敌方英雄 2 名以上且比身边友方…
 往哪走：只在墙上开门、穿到墙的另一边（英雄联盟的神奇旅程）：撤——背向身边敌人中心左右 75° 内、60000 内有墙的方向（20000 时他在线上只有 15% 的时间附近有墙，一局开不…
 队友：门边 25000 内的友方英雄一起穿过去（同样的位移；落点在墙里就落在他出口旁，再不行就不带）
@@ -10700,7 +10702,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>波比附加包（league_poppy v0.1.0）
+          <t>波比附加包（league_poppy v0.1.1）
 坚定风采的光环：光环里正在突进的敌方英雄被挡下：击飞 0.5 秒、受魔法伤害，然后缚地并减速 2 秒（每次光环每人一次）
 坚定风采的双抗：生命低于 40% 时翻倍
 英勇冲锋：撞到墙上（地图的墙格、5v5 地图的四边）才再受一次伤害并眩晕；没墙就只推开
@@ -11454,7 +11456,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.6）
+          <t>悠米附加包（league_yuumi v0.1.7）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11600,643 +11602,701 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
+          <t>荏妮</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Renni</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>tft_renni</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>链锯每次咬3下，每下造成42% 攻击力物理伤害。微光狂热：生命低于40%时注射微光（每30秒一次），4秒内攻速+40%，并回复20%最大生命。
+（攻击间隔 1.2 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>链锯冲撞：冲向目标，在前方扇形里锯3次，每次造成40 + 60% 攻击力物理伤害并减速30%，持续1.5秒。
+（冷却 9 秒 · 施放距离 40000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>锯刃格挡：竖起链锯格挡：获得100+80% 攻击力护盾，持续2.5秒，期间减伤20%。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>泥奔者重击：把目标挑起举过头顶，造成120 + 190% 攻击力物理伤害并击飞1.1秒，期间回复15%最大生命；再狠狠砸下，对前方周围敌人造成70 + 110% 攻击力物理伤害。
+（冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_renni.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
           <t>刀疤</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Scar</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_scar</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>长矛刺击造成100% 攻击力物理伤害。野火冲刺：每6秒下一击踩滑板冲刺，造成40 + 110% 攻击力+30% 法强伤害，回复上次冲刺以来所受伤害的25%。监察：生命不低于50%时减伤20%，否则10%。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>水坑狙击惊喜：向最近的3名敌人各扔一颗炸弹，造成70 + 80% 法强魔法伤害并晕眩1秒；自己回复60 + 60% 法强生命。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>长矛横扫：长矛横扫前方，造成50 + 80% 攻击力+2% 最大生命物理伤害并击退敌人。
 （冷却 9 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>野火突袭：踩滑板冲向敌人，途中丢下两颗燃烧弹（各40 + 40% 法强魔法伤害）；落地爆炸，周围敌人受到120 + 100% 法强魔法伤害并被击飞0.5秒，之后4秒内减伤40%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scar.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L186"/>
+  <autoFilter ref="A1:L187"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12423,6 +12483,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L187" r:id="rId186"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smeech: hero page, README table, previews; versions main 0.254.0 / league.dll 0.8.2 / illaoi 0.2.25 / sylas 0.2.25 / viego_soul 0.2.18 / yuumi 0.1.8 / tft 0.16.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$188</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L187"/>
+  <dimension ref="A1:L188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.24）
+          <t>俄洛伊附加包（league_illaoi v0.2.25）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -1720,7 +1720,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>克烈附加包（league_kled v0.1.0）
+          <t>克烈附加包（league_kled v0.1.1）
 斯嘎尔的血：本包自己记斯嘎尔的血：这条命第一次骑上 sk_hp + 攻击 sk_ad%，勇气满了重新骑上 re_hp + 攻击 re_ad%，骑着时受到的伤害从这里扣，扣完就让他下马
 捕熊夹的绳子：被夹住的英雄离克烈超过 q_break，绳子断，不拽
 下马的样子：整身步行：下马时站着、跑着、挨打和普攻第一帧都画步行的克烈</t>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.17）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.18）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -6313,7 +6313,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>加里奥附加包（league_galio v0.1.1）
+          <t>加里奥附加包（league_galio v0.1.2）
 主包 league 保持纯数据。用户选了「主包数据 + 附加包」。这个附加包用原生代码做主包数据做不到的三件事： - 杜朗护盾的被动护盾按「多久没挨打」给：主包里加里奥普攻时给护盾（每 12 秒最多一次），因为数据读不到「多久没受伤」。 附加包的被动 league_galio:colossus 记下他最后一次受伤的 tick，12 秒没受伤就给 90 + …</t>
         </is>
       </c>
@@ -7274,7 +7274,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.23）
+          <t>塞拉斯附加包（league_sylas v0.2.25）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11456,7 +11456,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.7）
+          <t>悠米附加包（league_yuumi v0.1.8）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11776,527 +11776,585 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
+          <t>史密奇</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Smeech</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>tft_smeech</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
+（攻击间隔 0.9 秒 · 攻击距离 23000）</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
+（冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
+（冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
+（冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L187"/>
+  <autoFilter ref="A1:L188"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12484,6 +12542,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L188" r:id="rId187"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Steb: hero page, README table, previews; card -9 by the rule; reels; versions main 0.256.0 / league.dll 0.8.4 / illaoi 0.2.27 / sylas 0.2.27 / viego_soul 0.2.20 / yuumi 0.1.10 / tft 0.18.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.26）
+          <t>俄洛伊附加包（league_illaoi v0.2.27）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.19）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.20）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7274,7 +7274,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.26）
+          <t>塞拉斯附加包（league_sylas v0.2.27）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11456,7 +11456,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.9）
+          <t>悠米附加包（league_yuumi v0.1.10）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12411,8 +12411,66 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>斯特卜</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Steb</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>tft_steb</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>辅助</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
+（攻击间隔 1.5 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
+（冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
+（冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
+（冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L189"/>
+  <autoFilter ref="A1:L190"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12602,6 +12660,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L187" r:id="rId186"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L188" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L190" r:id="rId189"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Taric PPU 1.55 registered: league.dll 0.8.6 (hd.rs row), main 0.258.0; Illaoi's spirit, Viego's souls (his hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.22; preview_taric on the dense frames; hero page, gallery, tech notes, README
40 game px as his 1x sprite: no SIZES row, the face point (-3, -38) stays (tfm2_ase face: PASS); his card keeps -10
(bp_card_audit: the rule's -10, top -29.3, Q's raised hand inside the canvas). The idle and ban/pick reels are
hero_reels' cuts of the new frames. Sylas's tables unchanged (he copies Taric's kit, not his frames).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.21）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.22）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -6000,9 +6000,9 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>阿兹尔附加包（league_azir v0.1.4）
+          <t>阿兹尔附加包（league_azir v0.1.5）
 太阳圆盘（并入被动，英雄联盟的「恕瑞玛的传承」）：开局记下我方每座塔；每局一次，某座塔倒了、阿兹尔走到废墟 d_near（60000）内、废墟 d_range（45000）内有敌人时，圆盘从沙里升起，立 d_life tick（…
-禁军之墙的禁军：按阿兹尔到大招目标的方向朝左或朝右（反推时他已经绕到目标身后，禁军就朝回冲）；伤害和击退还是数据那道墙的
+禁军之墙的禁军：按阿兹尔到大招目标的方向朝左或朝右（反推时他已经绕到目标身后，禁军就朝回冲）；伤害还是数据那道墙的。墙停下后再立 3 秒，敌方英雄走不过去；墙打中的敌人被带到墙停下的地方外面（正…
 沙兵（用户：「沙兵没攻击动作 你想办法补吧 不让codex了 还有不面向敌人」）：从侧面画：升起，之后每 ss_stand tick（4）盖一次站姿，朝 60 像素内最近的敌人（先英雄，敌人正好在它上下方时不转）；刺过以后下一次改放刺击（ss_stab tic…</t>
         </is>
       </c>
@@ -11334,7 +11334,7 @@
       <c r="I171" s="2" t="inlineStr"/>
       <c r="J171" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="K171" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Kayle PPU 2.29 registered: league.dll 0.8.8 (hd.rs row), main 0.259.0; her card 0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.23; preview_kayle / preview_kayle_ascend on the dense frames; hero page, gallery, tech notes, README
49 game px as her 1x sprite and hovering 2 px as before: no SIZES row, the face point (-2, -40) stays (tfm2_ase face:
PASS). Her card: -5 cut her wing tips (bp_card_audit CLIPPED, the rule's +1, never positive) -> 0, the wings whole in
the mock. The ascension's wing layers and halo sit behind the new body as before. The idle and ban/pick reels are
hero_reels' cuts of the new frames. Sylas's tables unchanged. Main merged first (Wukong 1.53 / dll 0.8.7, Tahm).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -1600,7 +1600,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.22）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.23）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）

</xml_diff>

<commit_message>
tft_idas: wired in - texts (5 languages), 16 sounds, champion_view, tft 0.20.0; rig (11 Codex poses, the open mouths kept crimson; the run a placeholder until Codex's run2), PPU 2.45 / HD; Illaoi's ghost, Viego/Neeko souls, Yuumi crowns (Kayle 38 -> 39: her current sheet), reels; hero page + README (support 30)
Sylas's copy waits for the effects (his steal-table test fails until then).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L191"/>
+  <dimension ref="A1:L192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6003,7 +6003,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>阿兹尔附加包（league_azir v0.1.5）
+          <t>阿兹尔附加包（league_azir v0.1.6）
 太阳圆盘（并入被动，英雄联盟的「恕瑞玛的传承」）：开局记下我方每座塔；每局一次，某座塔倒了、阿兹尔走到废墟 d_near（60000）内、废墟 d_range（45000）内有敌人时，圆盘从沙里升起，立 d_life tick（…
 禁军之墙的禁军：按阿兹尔到大招目标的方向朝左或朝右（反推时他已经绕到目标身后，禁军就朝回冲）；伤害还是数据那道墙的。墙停下后再立 3 秒，敌方英雄走不过去；墙打中的敌人被带到墙停下的地方外面（正…
 沙兵（用户：「沙兵没攻击动作 你想办法补吧 不让codex了 还有不面向敌人」）：从侧面画：升起，之后每 ss_stand tick（4）盖一次站姿，朝 60 像素内最近的敌人（先英雄，敌人正好在它上下方时不转）；刺过以后下一次改放刺击（ss_stab tic…</t>
@@ -12418,121 +12418,179 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
+          <t>艾达丝</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Idas</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>tft_idas</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>辅助</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
+（攻击间隔 1.4 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
+（冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
+（冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
+（冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L191"/>
+  <autoFilter ref="A1:L192"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12724,6 +12782,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L189" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L192" r:id="rId191"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: the add-on pages' versions (illaoi, sylas, viego, yuumi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.28）
+          <t>俄洛伊附加包（league_illaoi v0.2.29）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.25）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.26）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.28）
+          <t>塞拉斯附加包（league_sylas v0.2.29）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.12）
+          <t>悠米附加包（league_yuumi v0.1.13）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控

</xml_diff>

<commit_message>
tft_daeja: hero page (dev record), README table (ADC 27, tft 19), docs/heroes.xlsx, the add-on pages' versions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L192"/>
+  <dimension ref="A1:L193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.29）
+          <t>俄洛伊附加包（league_illaoi v0.2.30）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.26）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.27）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.29）
+          <t>塞拉斯附加包（league_sylas v0.2.30）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.13）
+          <t>悠米附加包（league_yuumi v0.1.14）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12361,237 +12361,295 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
+          <t>迭嘉</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>Daeja</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>tft_daeja</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>ADC</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
+（攻击间隔 1.2 秒 · 攻击距离 60000）</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
+（冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
+（冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
+（冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L192"/>
+  <autoFilter ref="A1:L193"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12784,6 +12842,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L191" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId192"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_shiohyu: hero page (dev record), README table (top 44, tft 20), docs/heroes.xlsx, the add-on pages' versions; versions main 0.262.0 / league.dll 0.8.15 / illaoi 0.2.31 (needs main 0.262.0) / sylas 0.2.31 / viego_soul 0.2.28 / yuumi 0.1.15 / tft 0.22.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L193"/>
+  <dimension ref="A1:L194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.30）
+          <t>俄洛伊附加包（league_illaoi v0.2.31）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.27）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.28）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.30）
+          <t>塞拉斯附加包（league_sylas v0.2.31）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.14）
+          <t>悠米附加包（league_yuumi v0.1.15）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11781,875 +11781,933 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
+          <t>石傲玉</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Shi Oh Yu</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>tft_shiohyu</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>左右爪交替挥击，第3下造成20 + 130% 攻击力物理伤害。玉石之肤：生命低于50%时化作玉石，减伤40%（3秒，冷却30秒）。
+（攻击间隔 1.1 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>玉拳连打：冲向目标连打4拳，每拳造成15 + 45% 攻击力物理伤害。
+（冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>震地：一拳砸地，周围敌人受到50 + 110% 攻击力物理伤害，被击飞0.75秒并减速35%。
+（冷却 9 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>玉龙形态：减伤35%、免疫控制，接下来3次普攻各造成40 + 175% 攻击力伤害：第1下晕眩1秒；第2下为真实伤害；第3下打出直线冲击波，晕眩沿线敌人。
+（冷却 25 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_shiohyu.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L193"/>
+  <autoFilter ref="A1:L194"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12843,6 +12901,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L191" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L192" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId193"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_syfen: hero page (dev record), README table (jungle 45, tft 21), docs/heroes.xlsx, the add-on pages' versions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L194"/>
+  <dimension ref="A1:L195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.31）
+          <t>俄洛伊附加包（league_illaoi v0.2.32）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.28）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.29）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.31）
+          <t>塞拉斯附加包（league_sylas v0.2.32）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.15）
+          <t>悠米附加包（league_yuumi v0.1.16）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11955,759 +11955,817 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
+          <t>赛芬</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Sy'fen</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>tft_syfen</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
+（攻击间隔 1 秒 · 攻击距离 30000）</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
+（冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
+（冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L194"/>
+  <autoFilter ref="A1:L195"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12902,6 +12960,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L192" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L195" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_sohm: hero page (dev record), README table (mid 49, tft 22), docs/heroes.xlsx, the add-on pages' versions; versions main 0.264.0 / league.dll 0.8.18 / illaoi 0.2.33 (needs main 0.264.0) / sylas 0.2.33 / viego_soul 0.2.30 / yuumi 0.1.17 / tft 0.24.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L195"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.32）
+          <t>俄洛伊附加包（league_illaoi v0.2.33）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.29）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.30）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7278,7 +7278,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.32）
+          <t>塞拉斯附加包（league_sylas v0.2.33）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11461,7 +11461,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.16）
+          <t>悠米附加包（league_yuumi v0.1.17）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12477,295 +12477,353 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
+          <t>索姆</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Sohm</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>tft_sohm</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>中单</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
+（攻击间隔 1.5 秒 · 攻击距离 55000）</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
+（冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
+（冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
+（冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L195"/>
+  <autoFilter ref="A1:L196"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -12961,6 +13019,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L196" r:id="rId195"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leona PPU 1.76 registered: league.dll 0.8.19 (hd.rs row), main 0.265.0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.31; preview_leona on the dense frames; hero page, gallery, tech notes, README
41 game px as her 1x sprite: no SIZES row, the face point (3, -35) stays (tfm2_ase face: PASS); her card keeps -10
(bp_card_audit flags only W1's raised sword tip, the head fits). The idle and ban/pick reels are hero_reels' cuts of the
new frames. Sylas's tables unchanged. Main merged first (dll 0.8.18 / main 0.264.0, as installed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.30）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.31）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -10278,7 +10278,7 @@
       <c r="I154" s="2" t="inlineStr"/>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Sona PPU 3.88 registered: league.dll 0.8.20 (hd.rs row), main 0.266.0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.32; preview_sona on the dense frames; hero page, gallery, tech notes, README
40 game px as her 1x sprite: no SIZES row, the face point (-1, -36) stays (tfm2_ase face: PASS); her card keeps -10
(bp_card_audit: no flag). The idle and ban/pick reels are hero_reels' cuts of the new frames. Sylas's tables
unchanged. ui_sheets: bp 200.5 / 768 MiB (her card 4.9). Main merged first (#627 Teemo; dll 0.8.19 / main 0.265.0).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.31）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.32）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -11155,7 +11155,7 @@
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="K168" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Briar PPU 2.94 registered: league.dll 0.8.21 (hd.rs row), main 0.267.0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.33; preview_briar on the dense frames; hero page, gallery, tech notes, README
46 game px as her 1x sprite: no SIZES row, the face point (-3, -34) stays (tfm2_ase face: PASS); her card -8 -> -3
(committed with the actions: the taller frames clipped the pillory's gem). The idle and ban/pick reels are
hero_reels' cuts of the new frames. Sylas's tables unchanged. ui_sheets ok. Main merged first (#629 Akshan; dll
0.8.20 / main 0.266.0 / viego 0.2.32, as installed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -3201,7 +3201,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.94</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.32）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.33）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）

</xml_diff>

<commit_message>
tft_terra: hero page (dev record), README table (top 45, tft 23, 196), docs/heroes.xlsx, the add-on pages' versions; versions main 0.269.0 / league.dll 0.8.22 / illaoi 0.2.34 (needs main 0.269.0) / sylas 0.2.34 / viego_soul 0.2.35 / yuumi 0.1.19 / tft 0.25.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L196"/>
+  <dimension ref="A1:L197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.33）
+          <t>俄洛伊附加包（league_illaoi v0.2.34）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.34）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.35）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7279,7 +7279,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.33）
+          <t>塞拉斯附加包（league_sylas v0.2.34）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.18）
+          <t>悠米附加包（league_yuumi v0.1.19）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11840,991 +11840,1049 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
+          <t>泰拉</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Terra</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>tft_terra</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>岩爪一拍，造成100% 攻击力物理伤害。巨岩之躯：受到的伤害永久减少18%。
+（攻击间隔 1.1 秒 · 攻击距离 30000）</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>裂地咬：低头扑咬目标，造成40 + 130% 攻击力 + 50% 护甲物理伤害（=护甲+魔抗），减速30%（1.5秒）。
+（冷却 8 秒 · 施放距离 34000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>龙威咆哮：仰天咆哮，嘲讽周围敌人1.5秒，自己获得80 + 80% 攻击力的岩石护盾（3秒）。
+（冷却 12 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>地震：重踏三次（施放中免疫控制），每踏对周围敌人造成30 + 70% 攻击力 + 32% 护甲物理伤害；之后护甲和魔抗+60（8秒）。
+（冷却 40 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_terra.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>赛芬</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Sy'fen</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_syfen</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
 （攻击间隔 1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
 （冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2.52</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>索姆</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Sohm</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_sohm</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
 （冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
 （冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
 （冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="2" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
+      <c r="C197" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="G197" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr">
+      <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="3" t="inlineStr">
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L196"/>
+  <autoFilter ref="A1:L197"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13021,6 +13079,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L195" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L197" r:id="rId196"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_sentinel: hero page (dev record), README table (jungle 46, tft 24, 197), docs/heroes.xlsx, previews, the add-on pages' versions; versions main 0.273.0 / league.dll 0.8.26 / illaoi 0.2.36 (needs main 0.273.0) / sylas 0.2.36 / viego_soul 0.2.37 / yuumi 0.1.21 / tft 0.27.0 (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L197"/>
+  <dimension ref="A1:L198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.34）
+          <t>俄洛伊附加包（league_illaoi v0.2.36）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.35）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.37）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7279,7 +7279,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.34）
+          <t>塞拉斯附加包（league_sylas v0.2.36）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.19）
+          <t>悠米附加包（league_yuumi v0.1.21）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11956,933 +11956,991 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
+          <t>苍蓝雕纹魔像</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>tft_sentinel</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>巨拳砸下，造成100% 攻击力物理伤害。蓝霸符：每放一个技能，身边友军的技能剩余冷却立刻降到最多67%。
+（攻击间隔 1.27 秒 · 攻击距离 26000）</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>双拳重砸：双拳砸地，对周围敌人造成85 + 105% 法强 + 4% 最大生命魔法伤害并减速30%（2秒）。
+（冷却 6.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>雕纹石肤：符文亮起，获得120 + 120% 法强护盾（4秒），嘲讽周围敌人1.2秒。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>蔚蓝冲击波：获得150 + 120% 法强护盾，猛砸地面，朝敌方英雄最多的方向裂开裂隙：击飞、170 + 170% 法强 + 4% 最大生命魔法伤害，破法（下一个技能晚2秒）。
+（冷却 50 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sentinel.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>赛芬</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Sy'fen</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_syfen</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
 （攻击间隔 1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
 （冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2.52</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>索姆</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Sohm</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_sohm</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
 （冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
 （冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
 （冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="2" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
+      <c r="C197" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="G197" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr">
+      <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="3" t="inlineStr">
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B197" s="2" t="inlineStr">
+      <c r="B198" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C197" s="2" t="inlineStr">
+      <c r="C198" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D198" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E197" s="2" t="inlineStr">
+      <c r="E198" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
+      <c r="F198" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G197" s="2" t="inlineStr">
+      <c r="G198" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H197" s="2" t="inlineStr">
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I197" s="2" t="inlineStr"/>
-      <c r="J197" s="2" t="inlineStr">
+      <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
-      <c r="L197" s="3" t="inlineStr">
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L197"/>
+  <autoFilter ref="A1:L198"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13080,6 +13138,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L195" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L196" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L198" r:id="rId197"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_brambleback: hero page (dev record), README table (jungle 48, tft 26, 199), docs/heroes.xlsx, previews, the add-on pages' versions; versions main 0.274.0 / league.dll 0.8.27 / illaoi 0.2.37 (needs main 0.274.0) / sylas 0.2.37 / viego_soul 0.2.38 / yuumi 0.1.22 / tft 0.28.0 (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L199"/>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.36）
+          <t>俄洛伊附加包（league_illaoi v0.2.37）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.37）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.38）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7279,7 +7279,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.36）
+          <t>塞拉斯附加包（league_sylas v0.2.37）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.21）
+          <t>悠米附加包（league_yuumi v0.1.22）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11898,1107 +11898,1165 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
+          <t>绯红印记树怪</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Brambleback</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>tft_brambleback</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>大爪横扫，造成100% 攻击力物理伤害。红霸符：普攻灼烧目标3秒（每秒1.2% 最大生命真实伤害），回复1.5%生命；击杀后扑向下一个敌人，造成60 + 120% 攻击力物理伤害。
+（攻击间隔 1.1 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>荆棘飞扑：跃起扑向目标，造成60 + 150% 攻击力物理伤害并减速30%（1秒）。
+（冷却 7 秒 · 施放距离 55000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>绯红咆哮：人立怒吼：周围敌人减速30%、攻击力降低20%，自己受到的伤害降低25%，持续3秒。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>猩红之怒：狂暴6秒：攻击力+55%、攻速+35%，无视目标40%护甲。
+（冷却 50 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_brambleback.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>苍蓝雕纹魔像</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Sentinel</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_sentinel</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>巨拳砸下，造成100% 攻击力物理伤害。蓝霸符：每放一个技能，身边友军的技能剩余冷却立刻降到最多67%。
 （攻击间隔 1.27 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>双拳重砸：双拳砸地，对周围敌人造成85 + 105% 法强 + 4% 最大生命魔法伤害并减速30%（2秒）。
 （冷却 6.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>雕纹石肤：符文亮起，获得120 + 120% 法强护盾（4秒），嘲讽周围敌人1.2秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>蔚蓝冲击波：获得150 + 120% 法强护盾，猛砸地面，朝敌方英雄最多的方向裂开裂隙：击飞、170 + 170% 法强 + 4% 最大生命魔法伤害，破法（下一个技能晚2秒）。
 （冷却 50 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sentinel.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>赛芬</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Sy'fen</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_syfen</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
 （攻击间隔 1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
 （冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2.52</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>呲呲</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Zippy</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_zippy</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>抬腿一蹬，造成100% 攻击力物理伤害。冒险家之魂：身边每有一个友方英雄，护甲和魔抗+10（最多4个）。
 （攻击间隔 0.97 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>后空翻踢：后空翻踢中目标，造成30 + 140% 攻击力物理伤害并击飞0.67秒。
 （冷却 7 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>翻滚冲锋：缩成羽毛球滚向敌人，路上的敌人受到40 + 80% 攻击力物理伤害；身边友方英雄移速+20%（2.5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>翻滚突袭：获得120 + 100% 攻击力护盾（2秒），跃起砸向生命百分比最高的敌方英雄（免疫控制），造成80 + 220% 攻击力物理伤害，晕眩1.5秒并略微击退。
 （冷却 40 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_zippy.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>索姆</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Sohm</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_sohm</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
 （冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
 （冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
 （冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="2" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
+      <c r="C197" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="G197" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr">
+      <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="3" t="inlineStr">
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B197" s="2" t="inlineStr">
+      <c r="B198" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C197" s="2" t="inlineStr">
+      <c r="C198" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D198" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E197" s="2" t="inlineStr">
+      <c r="E198" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
+      <c r="F198" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G197" s="2" t="inlineStr">
+      <c r="G198" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H197" s="2" t="inlineStr">
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I197" s="2" t="inlineStr"/>
-      <c r="J197" s="2" t="inlineStr">
+      <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
-      <c r="L197" s="3" t="inlineStr">
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="2" t="inlineStr">
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
+      <c r="B199" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C198" s="2" t="inlineStr">
+      <c r="C199" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D199" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E198" s="2" t="inlineStr">
+      <c r="E199" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F199" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G198" s="2" t="inlineStr">
+      <c r="G199" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H198" s="2" t="inlineStr">
+      <c r="H199" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I198" s="2" t="inlineStr"/>
-      <c r="J198" s="2" t="inlineStr">
+      <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K198" s="2" t="inlineStr"/>
-      <c r="L198" s="3" t="inlineStr">
+      <c r="K199" s="2" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="2" t="inlineStr">
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E200" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G199" s="2" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H199" s="2" t="inlineStr">
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr">
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L199"/>
+  <autoFilter ref="A1:L200"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13198,6 +13256,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L197" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L200" r:id="rId199"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_raptor: hero page (dev record), README table (ADC 28, tft 27, 200), docs/heroes.xlsx, previews, the add-on pages' versions; versions main 0.275.0 / league.dll 0.8.28 / illaoi 0.2.38 (needs main 0.275.0) / sylas 0.2.38 / viego_soul 0.2.39 / yuumi 0.1.23 / tft 0.29.0 (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L200"/>
+  <dimension ref="A1:L201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.37）
+          <t>俄洛伊附加包（league_illaoi v0.2.38）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.38）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.39）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7279,7 +7279,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.37）
+          <t>塞拉斯附加包（league_sylas v0.2.38）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.22）
+          <t>悠米附加包（league_yuumi v0.1.23）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12884,179 +12884,237 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
+          <t>深红锋喙鸟</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Mama Beak</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>tft_raptor</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>ADC</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>甩出一根锋羽，造成100% 攻击力物理伤害。橙霸符：它的物理伤害使目标护甲-6（3秒，最多5层）。
+（攻击间隔 1.17 秒 · 攻击距离 60000）</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>羽刃扇射：张开翅膀，扇形甩出5根羽刃，每根命中第一个敌人，造成35 + 55% 攻击力物理伤害。
+（冷却 6 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>惊飞跃退：受惊尖叫，往后一跳，之后3秒攻速+70%。
+（冷却 9 秒 · 施放距离 35000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>鸟群之家：召唤4只不可选中的小锋喙鸟（7秒）：它每次普攻，小鸟们一起啄同一目标，各造成18 + 30% 攻击力物理伤害。
+（冷却 45 秒 · 施放距离 65000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_raptor.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
+      <c r="B199" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C198" s="2" t="inlineStr">
+      <c r="C199" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D199" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E198" s="2" t="inlineStr">
+      <c r="E199" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F199" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G198" s="2" t="inlineStr">
+      <c r="G199" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H198" s="2" t="inlineStr">
+      <c r="H199" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I198" s="2" t="inlineStr"/>
-      <c r="J198" s="2" t="inlineStr">
+      <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K198" s="2" t="inlineStr"/>
-      <c r="L198" s="3" t="inlineStr">
+      <c r="K199" s="2" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="2" t="inlineStr">
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E200" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G199" s="2" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H199" s="2" t="inlineStr">
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr">
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B200" s="2" t="inlineStr">
+      <c r="B201" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D200" s="2" t="inlineStr">
+      <c r="D201" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
+      <c r="F201" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G200" s="2" t="inlineStr">
+      <c r="G201" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H200" s="2" t="inlineStr">
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I200" s="2" t="inlineStr"/>
-      <c r="J200" s="2" t="inlineStr">
+      <c r="I201" s="2" t="inlineStr"/>
+      <c r="J201" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="3" t="inlineStr">
+      <c r="K201" s="2" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L200"/>
+  <autoFilter ref="A1:L201"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13257,6 +13315,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L201" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Talon PPU 2.21 registered: league.dll 0.8.29 (hd.rs row), main 0.276.0; Illaoi's spirit, Viego's souls (his hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.40; preview_talon on the dense frames; hero page, gallery, tech notes, README. Leona's docs at PPU 1.5
39 game px as his 1x sprite: no SIZES row, the face point (10, -36) stays (tfm2_ase face: PASS); his card -1
(committed with the actions). The idle and ban/pick reels are hero_reels' cuts of the new frames. Sylas's tables
unchanged. ui_sheets ok, every add-on's override check ok. Main merged first (a446ce341, #642; dll 0.8.28 / main
0.275.0 / viego 0.2.39 as installed). Leona: README / hero page / tech notes 1.76 -> 1.5, her previews rerendered.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.39）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.40）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7479,7 +7479,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
@@ -10278,7 +10278,7 @@
       <c r="I154" s="2" t="inlineStr"/>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Thresh PPU 2.48 and Miss Fortune PPU 2.76 registered in the same release as Talon (league.dll 0.8.29, main 0.276.0, league_viego_soul 0.2.40 - none installed since): hd.rs rows, Illaoi's spirit, Viego's souls (their hd_ / lo_ tags); preview_thresh / preview_missfortune on the dense frames; hero pages, gallery, tech notes, README
40 / 38 game px as their 1x sprites: no SIZES rows, face points pass, cards as they were (Thresh -10, Miss Fortune
default). The idle and ban/pick reels are hero_reels' cuts of the new frames. Sylas's tables unchanged. ui_sheets ok,
every add-on's override check ok, cargo tests ok, league.dll builds. The user: 「动作通过」.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -9133,7 +9133,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.76</t>
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
@@ -11405,7 +11405,7 @@
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.48</t>
         </is>
       </c>
       <c r="K172" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
tft_elderdragon: hero page (dev record), README table (top 46, tft 28, 201), docs/heroes.xlsx, previews, the add-on pages' versions; versions main 0.279.0 / league.dll 0.8.32 / illaoi 0.2.39 (needs main 0.279.0) / sylas 0.2.39 / viego_soul 0.2.42 / yuumi 0.1.25 / neeko 0.1.2 / tft 0.30.0 (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L201"/>
+  <dimension ref="A1:L202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.38）
+          <t>俄洛伊附加包（league_illaoi v0.2.39）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5296,7 +5296,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.41）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.42）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7019,7 +7019,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>妮蔻附加包（league_neeko v0.1.1）
+          <t>妮蔻附加包（league_neeko v0.1.2）
 天生幻魅：脱战 2 秒后整个身体画成最近的友方英雄（站、跑、出招、挨打都用他的图）；放技能、被控（击飞、晕眩、禁锢、嘲讽、恐惧、魅惑、强制位移）、假扮以来挨了她 35% 最大生命的伤害、或…</t>
         </is>
       </c>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.38）
+          <t>塞拉斯附加包（league_sylas v0.2.39）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.24）
+          <t>悠米附加包（league_yuumi v0.1.25）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -11550,1571 +11550,1629 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
+          <t>远古巨龙</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Elder Dragon</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>tft_elderdragon</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>上单</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>撕咬目标，造成100% 攻击力物理伤害，目标身边的敌人受到35% 攻击力溅射。远古巨龙霸符：被它伤害后生命低于15%的敌方英雄直接被处决。
+（攻击间隔 1.2 秒 · 攻击距离 30000）</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>烈焰吐息：朝穿过目标、敌人最多的直线喷吐龙焰，造成70 + 130% 攻击力物理伤害，每烧过一人伤害-20%（最低40%），并引燃：3秒内每秒受到2.5%最大生命的物理伤害。
+（冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>龙翼风暴：立起身猛拍双翼，身边的敌人受到30 + 60% 攻击力物理伤害、被击退并减速35%（2秒），自己受到的伤害-25%。
+（冷却 10 秒 · 施放距离 25000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>绝伦火热：无敌飞上天空，1.5秒后砸落：大范围敌人受到80 + 80% 攻击力物理伤害、晕眩1.25秒并被引燃；获得30%全能吸血（5秒），立刻喷一次烈焰吐息。
+（冷却 60 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>2.84</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_elderdragon.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
           <t>可酷伯</t>
         </is>
       </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>Kobuko</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C176" s="2" t="inlineStr">
         <is>
           <t>tft_kobuko</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E175" s="2" t="inlineStr">
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>猫爪掌，造成100% 攻击力物理伤害。第二阶段：每条命第一次生命低于50%时进入狂怒，直到阵亡：攻击速度+40%、生命偷取20%。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>金爪真言：获得70 + 50% 法强的护盾（4秒）；4秒内下一次普攻变为金爪重掌，造成40 + 105% 攻击力 + 2%最大生命物理伤害并晕眩1秒。
 （冷却 9.5 秒 · 施放距离 25000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G175" s="2" t="inlineStr">
+      <c r="G176" s="2" t="inlineStr">
         <is>
           <t>猛虎扑：扑向目标，落地时周围的敌人受到40 + 70% 攻击力 + 2%最大生命物理伤害并被击飞0.4秒。
 （冷却 10.5 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H175" s="2" t="inlineStr">
+      <c r="H176" s="2" t="inlineStr">
         <is>
           <t>游戏结束！：一跃冲天（期间不可选中、免疫控制），砸落在敌方英雄身上：目标受到70 + 100% 攻击力 + 6%最大生命物理伤害，周围的敌人（含目标）再受到70 + 60% 攻击力 + 3%最大生命物理伤害并被击飞0.8秒。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="inlineStr">
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
-      <c r="L175" s="3" t="inlineStr">
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_kobuko.md</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
         <is>
           <t>荏妮</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Renni</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>tft_renni</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>链锯每次咬3下，每下造成42% 攻击力物理伤害。微光狂热：生命低于40%时注射微光（每30秒一次），4秒内攻速+40%，并回复20%最大生命。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>链锯冲撞：冲向目标，在前方扇形里锯3次，每次造成40 + 60% 攻击力物理伤害并减速30%，持续1.5秒。
 （冷却 9 秒 · 施放距离 40000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G176" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
         <is>
           <t>锯刃格挡：竖起链锯格挡：获得100+80% 攻击力护盾，持续2.5秒，期间减伤20%。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H177" s="2" t="inlineStr">
         <is>
           <t>泥奔者重击：把目标挑起举过头顶，造成120 + 190% 攻击力物理伤害并击飞1.1秒，期间回复15%最大生命；再狠狠砸下，对前方周围敌人造成70 + 110% 攻击力物理伤害。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr">
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="3" t="inlineStr">
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_renni.md</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>刀疤</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Scar</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
         <is>
           <t>tft_scar</t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E177" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>长矛刺击造成100% 攻击力物理伤害。野火冲刺：每6秒下一击踩滑板冲刺，造成40 + 110% 攻击力+30% 法强伤害，回复上次冲刺以来所受伤害的25%。监察：生命不低于50%时减伤20%，否则10%。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F177" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>水坑狙击惊喜：向最近的3名敌人各扔一颗炸弹，造成70 + 80% 法强魔法伤害并晕眩1秒；自己回复60 + 60% 法强生命。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G177" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>长矛横扫：长矛横扫前方，造成50 + 80% 攻击力+2% 最大生命物理伤害并击退敌人。
 （冷却 9 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H177" s="2" t="inlineStr">
+      <c r="H178" s="2" t="inlineStr">
         <is>
           <t>野火突袭：踩滑板冲向敌人，途中丢下两颗燃烧弹（各40 + 40% 法强魔法伤害）；落地爆炸，周围敌人受到120 + 100% 法强魔法伤害并被击飞0.5秒，之后4秒内减伤40%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I177" s="2" t="inlineStr"/>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="3" t="inlineStr">
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scar.md</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>塞薇卡</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Sevika</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>tft_sevika</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E178" s="2" t="inlineStr">
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>铁拳造成100% 攻击力物理伤害，每第3下钳击造成25 + 150% 攻击力。百变铁手：每次施放技能随机一个改件：火箭、护盾、35%攻速，12%中头奖强化本次技能。
 （攻击间隔 1.1 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F178" s="2" t="inlineStr">
+      <c r="F179" s="2" t="inlineStr">
         <is>
           <t>喷火器：喷火1.2秒，对前方扇形造成5次12 + 32% 攻击力物理伤害，期间减伤30%。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G178" s="2" t="inlineStr">
+      <c r="G179" s="2" t="inlineStr">
         <is>
           <t>伸缩拳：射出铁拳，造成40 + 120% 攻击力物理伤害并击退；撞到身后的敌人则两人眩晕1.2秒。
 （冷却 10 秒 · 施放距离 55000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H178" s="2" t="inlineStr">
+      <c r="H179" s="2" t="inlineStr">
         <is>
           <t>嚼一嚼：冲向目标连咬2口，每口60 + 135% 攻击力物理伤害，眩晕1.1秒并流血；目标生命低于15%时直接咬死，再冲向下一个英雄。
 （冷却 45 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="inlineStr">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="3" t="inlineStr">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sevika.md</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>石傲玉</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Shi Oh Yu</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>tft_shiohyu</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>左右爪交替挥击，第3下造成20 + 130% 攻击力物理伤害。玉石之肤：生命低于50%时化作玉石，减伤40%（3秒，冷却30秒）。
 （攻击间隔 1.1 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>玉拳连打：冲向目标连打4拳，每拳造成15 + 45% 攻击力物理伤害。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G179" s="2" t="inlineStr">
+      <c r="G180" s="2" t="inlineStr">
         <is>
           <t>震地：一拳砸地，周围敌人受到50 + 110% 攻击力物理伤害，被击飞0.75秒并减速35%。
 （冷却 9 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
+      <c r="H180" s="2" t="inlineStr">
         <is>
           <t>玉龙形态：减伤35%、免疫控制，接下来3次普攻各造成40 + 175% 攻击力伤害：第1下晕眩1秒；第2下为真实伤害；第3下打出直线冲击波，晕眩沿线敌人。
 （冷却 25 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I179" s="2" t="inlineStr"/>
-      <c r="J179" s="2" t="inlineStr">
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
         <is>
           <t>2.46</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="3" t="inlineStr">
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_shiohyu.md</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>泰拉</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>Terra</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>tft_terra</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>上单</t>
         </is>
       </c>
-      <c r="E180" s="2" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>岩爪一拍，造成100% 攻击力物理伤害。巨岩之躯：受到的伤害永久减少18%。
 （攻击间隔 1.1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>裂地咬：低头扑咬目标，造成40 + 130% 攻击力 + 50% 护甲物理伤害（=护甲+魔抗），减速30%（1.5秒）。
 （冷却 8 秒 · 施放距离 34000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G180" s="2" t="inlineStr">
+      <c r="G181" s="2" t="inlineStr">
         <is>
           <t>龙威咆哮：仰天咆哮，嘲讽周围敌人1.5秒，自己获得80 + 80% 攻击力的岩石护盾（3秒）。
 （冷却 12 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H180" s="2" t="inlineStr">
+      <c r="H181" s="2" t="inlineStr">
         <is>
           <t>地震：重踏三次（施放中免疫控制），每踏对周围敌人造成30 + 70% 攻击力 + 32% 护甲物理伤害；之后护甲和魔抗+60（8秒）。
 （冷却 40 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
-      <c r="J180" s="2" t="inlineStr">
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>1.45</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="3" t="inlineStr">
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_terra.md</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>绯红印记树怪</t>
         </is>
       </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Brambleback</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>tft_brambleback</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>大爪横扫，造成100% 攻击力物理伤害。红霸符：普攻灼烧目标3秒（每秒1.2% 最大生命真实伤害），回复1.5%生命；击杀后扑向下一个敌人，造成60 + 120% 攻击力物理伤害。
 （攻击间隔 1.1 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>荆棘飞扑：跃起扑向目标，造成60 + 150% 攻击力物理伤害并减速30%（1秒）。
 （冷却 7 秒 · 施放距离 55000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G181" s="2" t="inlineStr">
+      <c r="G182" s="2" t="inlineStr">
         <is>
           <t>绯红咆哮：人立怒吼：周围敌人减速30%、攻击力降低20%，自己受到的伤害降低25%，持续3秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H181" s="2" t="inlineStr">
+      <c r="H182" s="2" t="inlineStr">
         <is>
           <t>猩红之怒：狂暴6秒：攻击力+55%、攻速+35%，无视目标40%护甲。
 （冷却 50 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I181" s="2" t="inlineStr"/>
-      <c r="J181" s="2" t="inlineStr">
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="3" t="inlineStr">
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_brambleback.md</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>远古石甲虫</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Krug</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr">
         <is>
           <t>tft_krug</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E182" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>岩拳砸地，造成100% 攻击力物理伤害。碎岩重生：每条命第一次受到致命伤害时碎成石堆0.75秒，再以小石甲虫站起：生命35%、攻速+30%，嘲讽周围敌人1秒（至少隔60秒）。
 （攻击间隔 1.2 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr">
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>岩之摇滚：获得80 + 60% 法强的护盾（4秒），缩成石球滚向目标，造成40 + 140% 攻击力 + 6%最大生命物理伤害并击退。
 （冷却 8 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G182" s="2" t="inlineStr">
+      <c r="G183" s="2" t="inlineStr">
         <is>
           <t>坚岩外壳：缩进巨石2.5秒：护甲+40、魔抗+30；周围的敌人被嘲讽0.75秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H182" s="2" t="inlineStr">
+      <c r="H183" s="2" t="inlineStr">
         <is>
           <t>远古崩落：一跃而起（不可选中、免疫控制），砸进敌方英雄身边：周围敌人受到70 + 100% 攻击力 + 6%最大生命物理伤害并被击飞0.8秒；随后落石再造成40 + 4%最大生命物理伤害。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I182" s="2" t="inlineStr"/>
-      <c r="J182" s="2" t="inlineStr">
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="3" t="inlineStr">
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_krug.md</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
         <is>
           <t>苍蓝雕纹魔像</t>
         </is>
       </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Sentinel</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>tft_sentinel</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>巨拳砸下，造成100% 攻击力物理伤害。蓝霸符：每放一个技能，身边友军的技能剩余冷却立刻降到最多67%。
 （攻击间隔 1.27 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>双拳重砸：双拳砸地，对周围敌人造成85 + 105% 法强 + 4% 最大生命魔法伤害并减速30%（2秒）。
 （冷却 6.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G183" s="2" t="inlineStr">
+      <c r="G184" s="2" t="inlineStr">
         <is>
           <t>雕纹石肤：符文亮起，获得120 + 120% 法强护盾（4秒），嘲讽周围敌人1.2秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H183" s="2" t="inlineStr">
+      <c r="H184" s="2" t="inlineStr">
         <is>
           <t>蔚蓝冲击波：获得150 + 120% 法强护盾，猛砸地面，朝敌方英雄最多的方向裂开裂隙：击飞、170 + 170% 法强 + 4% 最大生命魔法伤害，破法（下一个技能晚2秒）。
 （冷却 50 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I183" s="2" t="inlineStr"/>
-      <c r="J183" s="2" t="inlineStr">
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="3" t="inlineStr">
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sentinel.md</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
         <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>赛芬</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Sy'fen</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_syfen</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
 （攻击间隔 1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
 （冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2.52</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>呲呲</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Zippy</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_zippy</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>抬腿一蹬，造成100% 攻击力物理伤害。冒险家之魂：身边每有一个友方英雄，护甲和魔抗+10（最多4个）。
 （攻击间隔 0.97 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>后空翻踢：后空翻踢中目标，造成30 + 140% 攻击力物理伤害并击飞0.67秒。
 （冷却 7 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>翻滚冲锋：缩成羽毛球滚向敌人，路上的敌人受到40 + 80% 攻击力物理伤害；身边友方英雄移速+20%（2.5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>翻滚突袭：获得120 + 100% 攻击力护盾（2秒），跃起砸向生命百分比最高的敌方英雄（免疫控制），造成80 + 220% 攻击力物理伤害，晕眩1.5秒并略微击退。
 （冷却 40 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_zippy.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>索姆</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Sohm</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_sohm</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
 （冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
 （冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
 （冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="2" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
+      <c r="C197" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="G197" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr">
+      <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="3" t="inlineStr">
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B197" s="2" t="inlineStr">
+      <c r="B198" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C197" s="2" t="inlineStr">
+      <c r="C198" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D198" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E197" s="2" t="inlineStr">
+      <c r="E198" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
+      <c r="F198" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G197" s="2" t="inlineStr">
+      <c r="G198" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H197" s="2" t="inlineStr">
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I197" s="2" t="inlineStr"/>
-      <c r="J197" s="2" t="inlineStr">
+      <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
-      <c r="L197" s="3" t="inlineStr">
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="2" t="inlineStr">
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
         <is>
           <t>深红锋喙鸟</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
+      <c r="B199" s="2" t="inlineStr">
         <is>
           <t>Mama Beak</t>
         </is>
       </c>
-      <c r="C198" s="2" t="inlineStr">
+      <c r="C199" s="2" t="inlineStr">
         <is>
           <t>tft_raptor</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D199" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E198" s="2" t="inlineStr">
+      <c r="E199" s="2" t="inlineStr">
         <is>
           <t>甩出一根锋羽，造成100% 攻击力物理伤害。橙霸符：它的物理伤害使目标护甲-6（3秒，最多5层）。
 （攻击间隔 1.17 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F199" s="2" t="inlineStr">
         <is>
           <t>羽刃扇射：张开翅膀，扇形甩出5根羽刃，每根命中第一个敌人，造成35 + 55% 攻击力物理伤害。
 （冷却 6 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G198" s="2" t="inlineStr">
+      <c r="G199" s="2" t="inlineStr">
         <is>
           <t>惊飞跃退：受惊尖叫，往后一跳，之后3秒攻速+70%。
 （冷却 9 秒 · 施放距离 35000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H198" s="2" t="inlineStr">
+      <c r="H199" s="2" t="inlineStr">
         <is>
           <t>鸟群之家：召唤4只不可选中的小锋喙鸟（7秒）：它每次普攻，小鸟们一起啄同一目标，各造成18 + 30% 攻击力物理伤害。
 （冷却 45 秒 · 施放距离 65000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I198" s="2" t="inlineStr"/>
-      <c r="J198" s="2" t="inlineStr">
+      <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr">
         <is>
           <t>1.56</t>
         </is>
       </c>
-      <c r="K198" s="2" t="inlineStr"/>
-      <c r="L198" s="3" t="inlineStr">
+      <c r="K199" s="2" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_raptor.md</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="2" t="inlineStr">
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E200" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G199" s="2" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H199" s="2" t="inlineStr">
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr">
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B200" s="2" t="inlineStr">
+      <c r="B201" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D200" s="2" t="inlineStr">
+      <c r="D201" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
+      <c r="F201" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G200" s="2" t="inlineStr">
+      <c r="G201" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H200" s="2" t="inlineStr">
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I200" s="2" t="inlineStr"/>
-      <c r="J200" s="2" t="inlineStr">
+      <c r="I201" s="2" t="inlineStr"/>
+      <c r="J201" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="3" t="inlineStr">
+      <c r="K201" s="2" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="2" t="inlineStr">
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B201" s="2" t="inlineStr">
+      <c r="B202" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
+      <c r="C202" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
+      <c r="D202" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E201" s="2" t="inlineStr">
+      <c r="E202" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr">
+      <c r="F202" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G201" s="2" t="inlineStr">
+      <c r="G202" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H201" s="2" t="inlineStr">
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I201" s="2" t="inlineStr"/>
-      <c r="J201" s="2" t="inlineStr">
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K201" s="2" t="inlineStr"/>
-      <c r="L201" s="3" t="inlineStr">
+      <c r="K202" s="2" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L201"/>
+  <autoFilter ref="A1:L202"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13316,6 +13374,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L202" r:id="rId201"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_murkwolf: hero page (dev record), README table (jungle 49, tft 29, 202), docs/heroes.xlsx, previews; versions main 0.281.0 / league.dll 0.8.34 / illaoi 0.2.40 (needs main 0.281.0) / sylas 0.2.40 / viego_soul 0.2.43 / yuumi 0.1.26 / neeko 0.1.3 / tft 0.31.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L202"/>
+  <dimension ref="A1:L203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.39）
+          <t>俄洛伊附加包（league_illaoi v0.2.40）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.42）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.43）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7020,7 +7020,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>妮蔻附加包（league_neeko v0.1.2）
+          <t>妮蔻附加包（league_neeko v0.1.3）
 天生幻魅：脱战 2 秒后整个身体画成最近的友方英雄（站、跑、出招、挨打都用他的图）；放技能、被控（击飞、晕眩、禁锢、嘲讽、恐惧、魅惑、强制位移）、假扮以来挨了她 35% 最大生命的伤害、或…</t>
         </is>
       </c>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.39）
+          <t>塞拉斯附加包（league_sylas v0.2.40）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.25）
+          <t>悠米附加包（league_yuumi v0.1.26）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12073,1107 +12073,1165 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
+          <t>暗影狼</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Murkwolf</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>tft_murkwolf</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>打野</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>两个头一起撕咬，造成100% 攻击力物理伤害。灰霸符：暴击率25%，随已损失生命值最多再+30%，技能也能暴击。
+（攻击间隔 0.93 秒 · 攻击距离 23000）</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>撕裂之爪：跃向附近生命值最低的敌人，造成40 + 110% 攻击力物理伤害。接下来3次攻击攻速+60%，额外造成10 + 30% 攻击力物理伤害。
+（冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>狂战士之嚎：仰头长嚎，5秒内吸血20%，伤害提高15%，对生命低于50%的敌人翻倍。
+（冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>狼群攻击：叫来2只小暗影狼扑向目标，造成40 + 60% 攻击力物理伤害。6秒内它每次攻击，小狼咬2口，每口12 + 25% 攻击力物理伤害。
+（冷却 45 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_murkwolf.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
           <t>苍蓝雕纹魔像</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>Sentinel</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C185" s="2" t="inlineStr">
         <is>
           <t>tft_sentinel</t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>巨拳砸下，造成100% 攻击力物理伤害。蓝霸符：每放一个技能，身边友军的技能剩余冷却立刻降到最多67%。
 （攻击间隔 1.27 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>双拳重砸：双拳砸地，对周围敌人造成85 + 105% 法强 + 4% 最大生命魔法伤害并减速30%（2秒）。
 （冷却 6.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G185" s="2" t="inlineStr">
         <is>
           <t>雕纹石肤：符文亮起，获得120 + 120% 法强护盾（4秒），嘲讽周围敌人1.2秒。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H184" s="2" t="inlineStr">
+      <c r="H185" s="2" t="inlineStr">
         <is>
           <t>蔚蓝冲击波：获得150 + 120% 法强护盾，猛砸地面，朝敌方英雄最多的方向裂开裂隙：击飞、170 + 170% 法强 + 4% 最大生命魔法伤害，破法（下一个技能晚2秒）。
 （冷却 50 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I184" s="2" t="inlineStr"/>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="3" t="inlineStr">
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sentinel.md</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>史密奇</t>
         </is>
       </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Smeech</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C186" s="2" t="inlineStr">
         <is>
           <t>tft_smeech</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>双爪轮流挥抓，造成100% 攻击力物理伤害。伏击专家：暴击率25%；技能也能暴击，技能暴击造成220%伤害。
 （攻击间隔 0.9 秒 · 攻击距离 23000）</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>废铁黑客：跳向范围内生命最低的敌人，连斩3次，每次造成25 + 70% 攻击力物理伤害；目标阵亡则再跳一次，伤害为70%。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G185" s="2" t="inlineStr">
+      <c r="G186" s="2" t="inlineStr">
         <is>
           <t>拆解：双爪撕扯目标，造成45 + 110% 攻击力物理伤害，并使其护甲降低30%，持续4秒。
 （冷却 8 秒 · 施放距离 26000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H185" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>废铁狂潮：1.2秒内不受控制、减伤30%，接连跳斩最多5名未被斩过的敌人，每次造成55 + 100% 攻击力物理伤害并获得10%暴击率（5秒）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I185" s="2" t="inlineStr"/>
-      <c r="J185" s="2" t="inlineStr">
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="K185" s="2" t="inlineStr"/>
-      <c r="L185" s="3" t="inlineStr">
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_smeech.md</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
         <is>
           <t>赛芬</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>Sy'fen</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>tft_syfen</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>翼爪和甩尾交替攻击，造成100% 攻击力物理伤害。幽影低语：他的伤害让敌人缩小4秒（护甲、魔抗-20%）；打缩小的敌人叠怒气，每层+5攻击力，最多5层。
 （攻击间隔 1 秒 · 攻击距离 30000）</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F187" s="2" t="inlineStr">
         <is>
           <t>噬咬：扑上去咬住目标，造成40 + 160% 攻击力物理伤害，无视33%护甲，回复30 + 30% 攻击力生命。
 （冷却 8 秒 · 施放距离 32000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G186" s="2" t="inlineStr">
+      <c r="G187" s="2" t="inlineStr">
         <is>
           <t>翼刃横扫：张开双翼横扫身边，造成40 + 100% 攻击力物理伤害并减速30%（1.5秒）。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H187" s="2" t="inlineStr">
         <is>
           <t>暴走：龙吼后冲向最远的敌方英雄（免疫控制），路上的敌人受到30 + 140% 攻击力物理伤害并晕眩1.25秒，最后猛咬一口造成60 + 235% 攻击力物理伤害，无视33%护甲。
 （冷却 40 秒 · 施放距离 72000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr">
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
         <is>
           <t>2.52</t>
         </is>
       </c>
-      <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="3" t="inlineStr">
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_syfen.md</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
         <is>
           <t>范德尔</t>
         </is>
       </c>
-      <c r="B187" s="2" t="inlineStr">
+      <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Vander</t>
         </is>
       </c>
-      <c r="C187" s="2" t="inlineStr">
+      <c r="C188" s="2" t="inlineStr">
         <is>
           <t>tft_vander</t>
         </is>
       </c>
-      <c r="D187" s="2" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E187" s="2" t="inlineStr">
+      <c r="E188" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。监察：受到的伤害降低10%，生命高于50%时降低20%。
 （攻击间隔 1.07 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
+      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>地下猎犬：摆出防御姿态，嘲讽周围的敌人0.75秒，获得40护甲和30魔抗（2.5秒）；下一拳造成40 + 140% 攻击力物理伤害，队里每有一个家人再加40% 攻击力。
 （冷却 10 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G187" s="2" t="inlineStr">
+      <c r="G188" s="2" t="inlineStr">
         <is>
           <t>铁拳突进：冲向敌人打出上勾拳，造成50 + 90% 攻击力物理伤害并晕眩0.5秒，身边的敌人受到35%的伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H187" s="2" t="inlineStr">
+      <c r="H188" s="2" t="inlineStr">
         <is>
           <t>桥头死守：跳进敌群砸地，周围的敌人受到150 + 150% 攻击力物理伤害并被击飞1秒；之后4秒内受到的伤害降低15%，身边每个敌方英雄再降低8%（最多4个）。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I187" s="2" t="inlineStr"/>
-      <c r="J187" s="2" t="inlineStr">
+      <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="3" t="inlineStr">
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_vander.md</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
         <is>
           <t>蔚奥莱</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="B189" s="2" t="inlineStr">
         <is>
           <t>Violet</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C189" s="2" t="inlineStr">
         <is>
           <t>tft_violet</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>挥拳造成100% 攻击力物理伤害。搏击手：每次命中额外造成5% 攻击力真实伤害，全能吸血10%；每条命第一次生命低于50%时，2秒内回复15%最大生命。
 （攻击间隔 0.93 秒 · 攻击距离 24000）</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>1-2-3连招：两记刺拳各造成50% 攻击力物理伤害，再一记上勾拳造成40 + 120% 攻击力物理伤害并击飞0.5秒。
 （冷却 8 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G188" s="2" t="inlineStr">
+      <c r="G189" s="2" t="inlineStr">
         <is>
           <t>冲拳：冲向敌人一拳打退，造成40 + 100% 攻击力物理伤害。
 （冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H188" s="2" t="inlineStr">
+      <c r="H189" s="2" t="inlineStr">
         <is>
           <t>底城怒拳：跳进敌群双拳砸地，周围的敌人受到120 + 130% 攻击力物理伤害并被击飞0.8秒；之后5秒内攻速+40%、吸血+5%，队里每有一个家人攻速再+10%。
 （冷却 50 秒 · 施放距离 50000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I188" s="2" t="inlineStr"/>
-      <c r="J188" s="2" t="inlineStr">
+      <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K188" s="2" t="inlineStr"/>
-      <c r="L188" s="3" t="inlineStr">
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_violet.md</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
         <is>
           <t>呲呲</t>
         </is>
       </c>
-      <c r="B189" s="2" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Zippy</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>tft_zippy</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>打野</t>
         </is>
       </c>
-      <c r="E189" s="2" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>抬腿一蹬，造成100% 攻击力物理伤害。冒险家之魂：身边每有一个友方英雄，护甲和魔抗+10（最多4个）。
 （攻击间隔 0.97 秒 · 攻击距离 26000）</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>后空翻踢：后空翻踢中目标，造成30 + 140% 攻击力物理伤害并击飞0.67秒。
 （冷却 7 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G189" s="2" t="inlineStr">
+      <c r="G190" s="2" t="inlineStr">
         <is>
           <t>翻滚冲锋：缩成羽毛球滚向敌人，路上的敌人受到40 + 80% 攻击力物理伤害；身边友方英雄移速+20%（2.5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H189" s="2" t="inlineStr">
+      <c r="H190" s="2" t="inlineStr">
         <is>
           <t>翻滚突袭：获得120 + 100% 攻击力护盾（2秒），跃起砸向生命百分比最高的敌方英雄（免疫控制），造成80 + 220% 攻击力物理伤害，晕眩1.5秒并略微击退。
 （冷却 40 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I189" s="2" t="inlineStr"/>
-      <c r="J189" s="2" t="inlineStr">
+      <c r="I190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="3" t="inlineStr">
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_zippy.md</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>拉露恩</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>Alune</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>tft_alune</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>把螺旋月环像飞盘一样甩出去，造成100% 攻击力物理伤害，月环飞回她手里，回程路上的敌人受到30% 攻击力物理伤害。月相：每放一次技能月亮长一档，最多3档；大招每档伤害+20%，砸完回到新月。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>月之降临：月光碎片从天而降，落在离她最近的3个敌人身上，每枚造成42 + 32% 法强魔法伤害，并使魔抗降低20%，持续6秒。
 （冷却 4.25 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
+      <c r="G191" s="2" t="inlineStr">
         <is>
           <t>月华：月光洒在她和身边的友方英雄身上，攻击速度提高36%，持续5秒。
 （冷却 10 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H190" s="2" t="inlineStr">
+      <c r="H191" s="2" t="inlineStr">
         <is>
           <t>月曜降临：敌方英雄脚下浮现月影，0.75秒后满月砸下：165 + 72% 法强魔法伤害×220%由范围内的敌人平分（每人最多180%），中心的敌人眩晕0.83秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I190" s="2" t="inlineStr"/>
-      <c r="J190" s="2" t="inlineStr">
+      <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="3" t="inlineStr">
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_alune.md</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>敖兴</t>
         </is>
       </c>
-      <c r="B191" s="2" t="inlineStr">
+      <c r="B192" s="2" t="inlineStr">
         <is>
           <t>Ao Shin</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>tft_aoshin</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E191" s="2" t="inlineStr">
+      <c r="E192" s="2" t="inlineStr">
         <is>
           <t>吐出球状闪电，造成100% 攻击力物理伤害。风暴龙威：交战3秒后天雷劈中周围所有敌方英雄，造成12%最大生命真实伤害并眩晕0.83秒；随后自身法术强度+30%（6秒，每20秒一次）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
         <is>
           <t>雷息：喷出一道雷息，直线上的敌人受到80 + 50% 法强魔法伤害并被沉默0.67秒。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
+      <c r="G192" s="2" t="inlineStr">
         <is>
           <t>腾云：驾云飞离附近的敌方英雄，获得110 + 40% 法强的风暴护盾（3秒）。
 （冷却 8 秒 · 施放距离 42000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H191" s="2" t="inlineStr">
+      <c r="H192" s="2" t="inlineStr">
         <is>
           <t>闪电暴雨：召来雷暴：12道闪电接连劈向周围随机的敌方英雄，每道造成55 + 32% 法强魔法伤害并沉默0.3秒。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I191" s="2" t="inlineStr"/>
-      <c r="J191" s="2" t="inlineStr">
+      <c r="I192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K191" s="2" t="inlineStr"/>
-      <c r="L191" s="3" t="inlineStr">
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_aoshin.md</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>诺姆希</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Nomsy</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C193" s="2" t="inlineStr">
         <is>
           <t>tft_nomsy</t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E192" s="2" t="inlineStr">
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>吐出小火团，造成100% 攻击力物理伤害。龙神之躯：生命值低于40%时每秒回复3%最大生命值。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>火球！：抛出大火球，爆炸造成90 + 63% 法强魔法伤害，再弹出2颗小火球打附近的敌人，各造成55%伤害。
 （冷却 4 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
+      <c r="G193" s="2" t="inlineStr">
         <is>
           <t>龙息：向前喷出扇形龙息，造成55 + 36% 法强魔法伤害并灼烧2秒，魔抗降低20%（4秒）。
 （冷却 7 秒 · 施放距离 45000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H192" s="2" t="inlineStr">
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>龙神飞升：飞上天空（减伤50%、免疫控制），降下10颗火球，各造成60 + 35% 法强魔法伤害；落地后攻速+30%、法强+25%（5秒）。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
-      <c r="J192" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="3" t="inlineStr">
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_nomsy.md</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>诺拉</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Norra</t>
         </is>
       </c>
-      <c r="C193" s="2" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>tft_norra</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E193" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>普攻100% 攻击力物理伤害。寄情琐物：每10秒技能落点撒3个琐物4秒，飞向踩到的敌方英雄：30 + 20% 法强魔法伤害并挂线缕；技能命中英雄冷却-20%。奇异旅程：贴身的敌人受40 + 30% 法强魔法伤害，放逐1.5秒后减速80%0.75秒。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>回忆涌现：蓄力后射出回忆魔法弹，自己后退一步：落点周围敌人受到35 + 28% 法强魔法伤害，已有线缕的英雄再受最大生命2%，随后挂上线缕；打中英雄时地上的琐物待爆：敌方英雄靠近就飞向他。
 （冷却 5.5 秒 · 施放距离 90000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>思乡线缕：在目标两侧打开两扇门，0.3秒后线缕穿过：范围内敌人受到35 + 26% 法强魔法伤害并挂上线缕：4秒内体型变大15%（更容易被命中），减速20%2秒。
 （冷却 10 秒 · 施放距离 85000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="H194" s="2" t="inlineStr">
         <is>
           <t>传送门欢腾！：在敌方英雄脚下展开大裂隙，每0.5秒一波共4波：两个毛线球沿一条穿过敌方英雄的线从两头对飞，路上敌人各受30 + 15% 法强魔法伤害，每个球碰到的第一个英雄减速80%0.5秒；第4波+40%。
 （冷却 50 秒 · 施放距离 100000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I193" s="2" t="inlineStr"/>
-      <c r="J193" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="3" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_norra.md</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
         <is>
           <t>爆爆</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>Powder</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>tft_powder</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>扔出自制小鞭炮，造成100% 攻击力物理伤害。伏击者：技能炸弹可以暴击（25%几率，伤害翻倍）。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>猴子炸弹：把上了发条的猴子炸弹丢到目标脚下，范围内敌人受到36 + 28% 法强魔法伤害，中心再受一次；被炸到的敌人灼烧3秒，并重伤4秒（受到治疗-40%）。
 （冷却 5.5 秒 · 施放距离 70000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G194" s="2" t="inlineStr">
+      <c r="G195" s="2" t="inlineStr">
         <is>
           <t>快跑，爆爆！：敌方英雄靠近时摔下闪光烟雾弹：周围敌人受到45 + 30% 法强魔法伤害并致盲1秒（无法普攻），自己向后跳开。
 （冷却 10 秒 · 施放距离 24000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="H195" s="2" t="inlineStr">
         <is>
           <t>海克斯水晶炸弹：把装着海克斯水晶的包丢向敌方英雄，引线烧完0.9秒后蓝光大爆炸：范围内敌人受到170 + 65% 法强魔法伤害并击飞0.75秒。
 （冷却 50 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr"/>
-      <c r="J194" s="2" t="inlineStr">
+      <c r="I195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
-      <c r="L194" s="3" t="inlineStr">
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_powder.md</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>希尔科</t>
         </is>
       </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Silco</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>tft_silco</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>甩出一支微光药剂，造成100% 攻击力物理伤害。统领：每次出生获得120 + 40% 法强护盾（15秒）；每放一次技能法强+10%，最多5层，阵亡清空。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>罐装畸变体：扔出储罐，造成65 + 45% 法强魔法伤害，放出2只畸变体扑向附近的敌人，各咬5口，每口15 + 11% 法强魔法伤害；被咬的人倒下就跳到下一个。
 （冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>微光注射：把微光抛给身边攻击力最高的友方英雄（没有就自己）：攻速+50%、移速+20%，4秒；药效过去扣当前生命的8%。
 （冷却 12 秒 · 施放距离 60000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H195" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>炼金狂潮：向敌方英雄扔出巨型储罐，造成180 + 80% 法强魔法伤害，放出4只畸变体，留下4秒毒雾：敌人减速30%，每秒受到6 + 4% 法强魔法伤害。
 （冷却 50 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr">
+      <c r="I196" s="2" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="3" t="inlineStr">
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_silco.md</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="2" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
         <is>
           <t>索姆</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B197" s="2" t="inlineStr">
         <is>
           <t>Sohm</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
+      <c r="C197" s="2" t="inlineStr">
         <is>
           <t>tft_sohm</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>中单</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>吐出水泡弹，造成100% 攻击力物理伤害。碧波之力：每次施放技能叠一层潮水（6秒，最多5层），每层法强+9%、攻速+9%。
 （攻击间隔 1.5 秒 · 攻击距离 55000）</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>潮涌：朝没开花的敌人冲出一道潮涌，沿途敌人受到95 + 65% 法强魔法伤害，目标头上开出水之花（15秒）；带花的敌人倒下，花跳到附近的敌人。
 （冷却 4 秒 · 施放距离 62000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="G197" s="2" t="inlineStr">
         <is>
           <t>海潮护佑：给附近生命比例最低的队友套上95 + 65% 法强的水盾（3秒），攻速+25%。
 （冷却 8 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H197" s="2" t="inlineStr">
         <is>
           <t>潮汐绽放：所有水之花一齐绽放，每朵花周围的敌人受到180 + 90% 法强魔法伤害，花随之散去；没有花时在目标身上绽放。
 （冷却 35 秒 · 施放距离 70000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I196" s="2" t="inlineStr"/>
-      <c r="J196" s="2" t="inlineStr">
+      <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="3" t="inlineStr">
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sohm.md</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
         <is>
           <t>迭嘉</t>
         </is>
       </c>
-      <c r="B197" s="2" t="inlineStr">
+      <c r="B198" s="2" t="inlineStr">
         <is>
           <t>Daeja</t>
         </is>
       </c>
-      <c r="C197" s="2" t="inlineStr">
+      <c r="C198" s="2" t="inlineStr">
         <is>
           <t>tft_daeja</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D198" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E197" s="2" t="inlineStr">
+      <c r="E198" s="2" t="inlineStr">
         <is>
           <t>推出风弹，造成100% 攻击力物理伤害。三连弹幕：每次普攻再射出3颗小风弹，各造成10 + 15% 法强魔法伤害，魔抗-4（3秒，可叠加）。
 （攻击间隔 1.2 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
+      <c r="F198" s="2" t="inlineStr">
         <is>
           <t>罡风轰击：双翼前扫，朝敌人最多的直线轰出穿透的风波，造成110 + 70% 法强魔法伤害。
 （冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G197" s="2" t="inlineStr">
+      <c r="G198" s="2" t="inlineStr">
         <is>
           <t>振翼退风：振翅朝身边的敌人扇出一阵风，造成40 + 30% 法强魔法伤害并减速40%（1.5秒），自己借风后跳。
 （冷却 10 秒 · 施放距离 40000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H197" s="2" t="inlineStr">
+      <c r="H198" s="2" t="inlineStr">
         <is>
           <t>苍穹罡风：展翅飞起（减伤30%、免疫控制），朝敌人最多的直线连续轰出3道大冲击波，各造成150 + 70% 法强魔法伤害。
 （冷却 45 秒 · 施放距离 75000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I197" s="2" t="inlineStr"/>
-      <c r="J197" s="2" t="inlineStr">
+      <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
-      <c r="L197" s="3" t="inlineStr">
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_daeja.md</t>
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="2" t="inlineStr">
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
         <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
+      <c r="B199" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C198" s="2" t="inlineStr">
+      <c r="C199" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D199" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E198" s="2" t="inlineStr">
+      <c r="E199" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
+      <c r="F199" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G198" s="2" t="inlineStr">
+      <c r="G199" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H198" s="2" t="inlineStr">
+      <c r="H199" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I198" s="2" t="inlineStr"/>
-      <c r="J198" s="2" t="inlineStr">
+      <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K198" s="2" t="inlineStr"/>
-      <c r="L198" s="3" t="inlineStr">
+      <c r="K199" s="2" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="2" t="inlineStr">
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>深红锋喙鸟</t>
         </is>
       </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Mama Beak</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>tft_raptor</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E200" s="2" t="inlineStr">
         <is>
           <t>甩出一根锋羽，造成100% 攻击力物理伤害。橙霸符：它的物理伤害使目标护甲-6（3秒，最多5层）。
 （攻击间隔 1.17 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>羽刃扇射：张开翅膀，扇形甩出5根羽刃，每根命中第一个敌人，造成35 + 55% 攻击力物理伤害。
 （冷却 6 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G199" s="2" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr">
         <is>
           <t>惊飞跃退：受惊尖叫，往后一跳，之后3秒攻速+70%。
 （冷却 9 秒 · 施放距离 35000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H199" s="2" t="inlineStr">
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>鸟群之家：召唤4只不可选中的小锋喙鸟（7秒）：它每次普攻，小鸟们一起啄同一目标，各造成18 + 30% 攻击力物理伤害。
 （冷却 45 秒 · 施放距离 65000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr">
         <is>
           <t>1.56</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr">
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_raptor.md</t>
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B200" s="2" t="inlineStr">
+      <c r="B201" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D200" s="2" t="inlineStr">
+      <c r="D201" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
+      <c r="F201" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G200" s="2" t="inlineStr">
+      <c r="G201" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H200" s="2" t="inlineStr">
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I200" s="2" t="inlineStr"/>
-      <c r="J200" s="2" t="inlineStr">
+      <c r="I201" s="2" t="inlineStr"/>
+      <c r="J201" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="3" t="inlineStr">
+      <c r="K201" s="2" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="2" t="inlineStr">
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B201" s="2" t="inlineStr">
+      <c r="B202" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
+      <c r="C202" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
+      <c r="D202" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E201" s="2" t="inlineStr">
+      <c r="E202" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr">
+      <c r="F202" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G201" s="2" t="inlineStr">
+      <c r="G202" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H201" s="2" t="inlineStr">
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I201" s="2" t="inlineStr"/>
-      <c r="J201" s="2" t="inlineStr">
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K201" s="2" t="inlineStr"/>
-      <c r="L201" s="3" t="inlineStr">
+      <c r="K202" s="2" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="2" t="inlineStr">
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
+      <c r="B203" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C202" s="2" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E202" s="2" t="inlineStr">
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
+      <c r="F203" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G202" s="2" t="inlineStr">
+      <c r="G203" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H202" s="2" t="inlineStr">
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I202" s="2" t="inlineStr"/>
-      <c r="J202" s="2" t="inlineStr">
+      <c r="I203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="3" t="inlineStr">
+      <c r="K203" s="2" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L202"/>
+  <autoFilter ref="A1:L203"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13376,6 +13434,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L203" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_meepsie: hero page (dev record), README table (support 31, tft 29, 202), docs/heroes.xlsx, previews, the add-on pages' versions; versions main 0.281.0 / league.dll 0.8.34 / illaoi 0.2.40 (needs main 0.281.0) / sylas 0.2.40 / viego_soul 0.2.43 / yuumi 0.1.26 / tft 0.31.0 (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L202"/>
+  <dimension ref="A1:L203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.39）
+          <t>俄洛伊附加包（league_illaoi v0.2.40）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.42）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.43）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.39）
+          <t>塞拉斯附加包（league_sylas v0.2.40）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.25）
+          <t>悠米附加包（league_yuumi v0.1.26）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -13117,63 +13117,121 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
+          <t>小木灵</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Meepsie</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>tft_meepsie</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>辅助</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>挥出月岩重拳，造成100% 攻击力物理伤害。木灵驾驶员：每一拳额外造成15 + 25% 法强魔法伤害。
+（攻击间隔 1.5 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>月尘震地：一拳砸向前方地面，扇形范围内的敌人受到100 + 70% 法强魔法伤害并减速40%（2秒）。
+（冷却 6 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>治疗木灵：驾驶员一招手，4只小木灵飞向身边生命比例最低的队友（名额有剩时也治疗自己），每0.5秒回复20 + 10% 法强生命，持续3秒。
+（冷却 9 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>宇宙大爆炸：跳向附近敌方英雄最多的地方砸地，周围的敌人受到160 + 90% 法强魔法伤害，离中心每远一格少35%；离落点最近的3个敌方英雄被击飞1.25秒。
+（冷却 35 秒 · 施放距离 45000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_meepsie.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
+      <c r="B203" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C202" s="2" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E202" s="2" t="inlineStr">
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
+      <c r="F203" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G202" s="2" t="inlineStr">
+      <c r="G203" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H202" s="2" t="inlineStr">
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I202" s="2" t="inlineStr"/>
-      <c r="J202" s="2" t="inlineStr">
+      <c r="I203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="3" t="inlineStr">
+      <c r="K203" s="2" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L202"/>
+  <autoFilter ref="A1:L203"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13376,6 +13434,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L203" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Murk Wolf: versions above Meepsie's (PR #649, installed with the same numbers): main 0.282.0 / league.dll 0.8.35 / illaoi 0.2.41 (needs main 0.282.0) / sylas 0.2.41 / viego_soul 0.2.44 / yuumi 0.1.27 / tft 0.32.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.40）
+          <t>俄洛伊附加包（league_illaoi v0.2.41）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.43）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.44）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.40）
+          <t>塞拉斯附加包（league_sylas v0.2.41）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.26）
+          <t>悠米附加包（league_yuumi v0.1.27）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控

</xml_diff>

<commit_message>
tft_scuttlecrab: hero page (dev record), README table (support 32, tft 31, 204), docs/heroes.xlsx, previews; hd.rs PPU written 2.667 (the docs read decimals) (「可以，继续收尾」)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$205</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L204"/>
+  <dimension ref="A1:L205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.41）
+          <t>俄洛伊附加包（league_illaoi v0.2.42）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.44）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.45）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.41）
+          <t>塞拉斯附加包（league_sylas v0.2.42）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -8172,7 +8172,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>佐伊附加包（league_zoe v0.4.0）
+          <t>佐伊附加包（league_zoe v0.5.0）
 催眠气泡的睡眠：一样是官方睡眠，2.25 秒（英雄联盟的时长）；睡着时头上有睡泡，醒了就摘掉，被打醒的放醒来的画面
 飞星的伤害：按真实飞行距离：出手点 20000 以内 100%，到 85000 线性加到 250%
 窃法巧手：另外：敌方英雄放大招时原地掉下一块法术碎片（20 秒，最多 3 块），她走到 18000 以内就捡起来，射 3 颗飞弹（打 70000 内最近的敌方英雄，每颗 45 + 15% …
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.27）
+          <t>悠米附加包（league_yuumi v0.1.28）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -13233,63 +13233,121 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
+          <t>迅捷蟹</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Scuttle Crab</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>tft_scuttlecrab</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>辅助</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>跳一段螃蟹舞，踩中身边所有敌人，造成100% 攻击力物理伤害。绿霸符：附近的友方英雄生命低于40%时回复12%最大生命（每人10秒一次）。
+（攻击间隔 1.33 秒 · 攻击距离 25000）</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>疾行神龛：在脚下放下神龛（4秒），水花使周围敌人受到80 + 60% 法强魔法伤害并减速40%；神龛里的友方英雄移速+30%、攻速+25%。
+（冷却 7 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>蟹壳护盾：缩进壳里，获得120 + 60% 法强护盾（2秒）。护盾打光或到时间时蟹壳碎裂：周围敌人受到80 + 60% 法强魔法伤害、眩晕0.5秒并减速40%。
+（冷却 6 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>你挖得动吗？：钻入地下2.5秒：受到的伤害降低50%、免疫控制，持续回复250 + 80% 法强生命；然后钻出地面，周围敌人受到160 + 60% 攻击力物理伤害并被击飞1.5秒。
+（冷却 25 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr"/>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr"/>
+      <c r="L204" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scuttlecrab.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B204" s="2" t="inlineStr">
+      <c r="B205" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C204" s="2" t="inlineStr">
+      <c r="C205" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D204" s="2" t="inlineStr">
+      <c r="D205" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E204" s="2" t="inlineStr">
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F204" s="2" t="inlineStr">
+      <c r="F205" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G204" s="2" t="inlineStr">
+      <c r="G205" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H204" s="2" t="inlineStr">
+      <c r="H205" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I204" s="2" t="inlineStr"/>
-      <c r="J204" s="2" t="inlineStr">
+      <c r="I205" s="2" t="inlineStr"/>
+      <c r="J205" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K204" s="2" t="inlineStr"/>
-      <c r="L204" s="3" t="inlineStr">
+      <c r="K205" s="2" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L204"/>
+  <autoFilter ref="A1:L205"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13494,6 +13552,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L205" r:id="rId204"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tft_gromp: hero page (dev record), README table (ADC 29, tft 32, 205), docs/heroes.xlsx, previews; league_* pages' versions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$206</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L205"/>
+  <dimension ref="A1:L206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.42）
+          <t>俄洛伊附加包（league_illaoi v0.2.43）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.45）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.46）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7020,7 +7020,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>妮蔻附加包（league_neeko v0.1.3）
+          <t>妮蔻附加包（league_neeko v0.1.4）
 天生幻魅：脱战 2 秒后整个身体画成最近的友方英雄（站、跑、出招、挨打都用他的图）；放技能、被控（击飞、晕眩、禁锢、嘲讽、恐惧、魅惑、强制位移）、假扮以来挨了她 35% 最大生命的伤害、或…</t>
         </is>
       </c>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.42）
+          <t>塞拉斯附加包（league_sylas v0.2.43）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.1.28）
+          <t>悠米附加包（league_yuumi v0.1.29）
 附身多久：不限时，队友死了才跳下来
 附身时能不能出招：能：Q、R、再给他一次旺盛精力，都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -12943,411 +12943,469 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
+          <t>魔沼蛙</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Gromp</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>tft_gromp</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>ADC</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>吐出毒口水，造成100% 攻击力物理伤害和40% 法强魔法伤害。紫霸符：战斗中每4秒法术加成+8，最多8层。
+（攻击间隔 1.2 秒 · 攻击距离 60000）</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>打嗝泡泡：打出一个毒泡泡，碰到第一个敌人造成110 + 80% 法强魔法伤害并炸开，周围敌人3秒内受到80 + 60% 法强魔法伤害。
+（冷却 5 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>黏液沼泽：往敌人脚下吐一滩黏液，持续4秒，站在里面的敌人减速55%，每秒受到24 + 16% 法强魔法伤害。
+（冷却 8 秒 · 施放距离 60000 · 施放：地点 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>毒沼大嗝：肚子鼓起变大5秒（受到伤害-20%），向前打出大嗝，造成170 + 80% 法强魔法伤害并减速35%，毒雾留在地上4秒，每秒36 + 21% 法强魔法伤害。
+（冷却 40 秒 · 施放距离 60000 · 施放：地点 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>1.69</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_gromp.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
           <t>麦迪</t>
         </is>
       </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Maddie</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>tft_maddie</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E200" s="2" t="inlineStr">
         <is>
           <t>步枪射击，造成100% 攻击力物理伤害。狙神：目标离得越远，她造成的伤害越高，最多+25%；被通缉的敌人阵亡时她领一份赏金：攻速+15%，最多4份。
 （攻击间隔 1.1 秒 · 攻击距离 68000）</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>连拨击锤：半蹲朝范围内最远的敌人连开6枪（先打英雄），每枪打中路上第一个敌人，造成10 + 40% 攻击力物理伤害。
 （冷却 9 秒 · 施放距离 80000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G199" s="2" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近当前生命最高的敌方英雄8秒：它受到的伤害+15%。
 （冷却 15 秒 · 施放距离 90000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H199" s="2" t="inlineStr">
+      <c r="H200" s="2" t="inlineStr">
         <is>
           <t>执法狙杀：瞄准后向生命比例最低的敌方英雄射出一发穿透子弹，路上每个敌人受到220 + 140% 攻击力物理伤害，按其已损失生命比例最多再加60%。
 （冷却 50 秒 · 施放距离 200000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I199" s="2" t="inlineStr"/>
-      <c r="J199" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
-      <c r="L199" s="3" t="inlineStr">
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_maddie.md</t>
         </is>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
         <is>
           <t>深红锋喙鸟</t>
         </is>
       </c>
-      <c r="B200" s="2" t="inlineStr">
+      <c r="B201" s="2" t="inlineStr">
         <is>
           <t>Mama Beak</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
+      <c r="C201" s="2" t="inlineStr">
         <is>
           <t>tft_raptor</t>
         </is>
       </c>
-      <c r="D200" s="2" t="inlineStr">
+      <c r="D201" s="2" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>甩出一根锋羽，造成100% 攻击力物理伤害。橙霸符：它的物理伤害使目标护甲-6（3秒，最多5层）。
 （攻击间隔 1.17 秒 · 攻击距离 60000）</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
+      <c r="F201" s="2" t="inlineStr">
         <is>
           <t>羽刃扇射：张开翅膀，扇形甩出5根羽刃，每根命中第一个敌人，造成35 + 55% 攻击力物理伤害。
 （冷却 6 秒 · 施放距离 60000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G200" s="2" t="inlineStr">
+      <c r="G201" s="2" t="inlineStr">
         <is>
           <t>惊飞跃退：受惊尖叫，往后一跳，之后3秒攻速+70%。
 （冷却 9 秒 · 施放距离 35000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H200" s="2" t="inlineStr">
+      <c r="H201" s="2" t="inlineStr">
         <is>
           <t>鸟群之家：召唤4只不可选中的小锋喙鸟（7秒）：它每次普攻，小鸟们一起啄同一目标，各造成18 + 30% 攻击力物理伤害。
 （冷却 45 秒 · 施放距离 65000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I200" s="2" t="inlineStr"/>
-      <c r="J200" s="2" t="inlineStr">
+      <c r="I201" s="2" t="inlineStr"/>
+      <c r="J201" s="2" t="inlineStr">
         <is>
           <t>1.56</t>
         </is>
       </c>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="3" t="inlineStr">
+      <c r="K201" s="2" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_raptor.md</t>
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="2" t="inlineStr">
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
         <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B201" s="2" t="inlineStr">
+      <c r="B202" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
+      <c r="C202" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
+      <c r="D202" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E201" s="2" t="inlineStr">
+      <c r="E202" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr">
+      <c r="F202" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G201" s="2" t="inlineStr">
+      <c r="G202" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H201" s="2" t="inlineStr">
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I201" s="2" t="inlineStr"/>
-      <c r="J201" s="2" t="inlineStr">
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K201" s="2" t="inlineStr"/>
-      <c r="L201" s="3" t="inlineStr">
+      <c r="K202" s="2" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="2" t="inlineStr">
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
+      <c r="B203" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C202" s="2" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E202" s="2" t="inlineStr">
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
+      <c r="F203" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G202" s="2" t="inlineStr">
+      <c r="G203" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H202" s="2" t="inlineStr">
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I202" s="2" t="inlineStr"/>
-      <c r="J202" s="2" t="inlineStr">
+      <c r="I203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="3" t="inlineStr">
+      <c r="K203" s="2" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="2" t="inlineStr">
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
         <is>
           <t>小木灵</t>
         </is>
       </c>
-      <c r="B203" s="2" t="inlineStr">
+      <c r="B204" s="2" t="inlineStr">
         <is>
           <t>Meepsie</t>
         </is>
       </c>
-      <c r="C203" s="2" t="inlineStr">
+      <c r="C204" s="2" t="inlineStr">
         <is>
           <t>tft_meepsie</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
+      <c r="D204" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E203" s="2" t="inlineStr">
+      <c r="E204" s="2" t="inlineStr">
         <is>
           <t>挥出月岩重拳，造成100% 攻击力物理伤害。木灵驾驶员：每一拳额外造成15 + 25% 法强魔法伤害。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F203" s="2" t="inlineStr">
+      <c r="F204" s="2" t="inlineStr">
         <is>
           <t>月尘震地：一拳砸向前方地面，扇形范围内的敌人受到100 + 70% 法强魔法伤害并减速40%（2秒）。
 （冷却 6 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G203" s="2" t="inlineStr">
+      <c r="G204" s="2" t="inlineStr">
         <is>
           <t>治疗木灵：驾驶员一招手，4只小木灵飞向身边生命比例最低的队友（名额有剩时也治疗自己），每0.5秒回复20 + 10% 法强生命，持续3秒。
 （冷却 9 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H203" s="2" t="inlineStr">
+      <c r="H204" s="2" t="inlineStr">
         <is>
           <t>宇宙大爆炸：跳向附近敌方英雄最多的地方砸地，周围的敌人受到160 + 90% 法强魔法伤害，离中心每远一格少35%；离落点最近的3个敌方英雄被击飞1.25秒。
 （冷却 35 秒 · 施放距离 45000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I203" s="2" t="inlineStr"/>
-      <c r="J203" s="2" t="inlineStr">
+      <c r="I204" s="2" t="inlineStr"/>
+      <c r="J204" s="2" t="inlineStr">
         <is>
           <t>2.88</t>
         </is>
       </c>
-      <c r="K203" s="2" t="inlineStr"/>
-      <c r="L203" s="3" t="inlineStr">
+      <c r="K204" s="2" t="inlineStr"/>
+      <c r="L204" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_meepsie.md</t>
         </is>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="2" t="inlineStr">
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
         <is>
           <t>迅捷蟹</t>
         </is>
       </c>
-      <c r="B204" s="2" t="inlineStr">
+      <c r="B205" s="2" t="inlineStr">
         <is>
           <t>Scuttle Crab</t>
         </is>
       </c>
-      <c r="C204" s="2" t="inlineStr">
+      <c r="C205" s="2" t="inlineStr">
         <is>
           <t>tft_scuttlecrab</t>
         </is>
       </c>
-      <c r="D204" s="2" t="inlineStr">
+      <c r="D205" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E204" s="2" t="inlineStr">
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>跳一段螃蟹舞，踩中身边所有敌人，造成100% 攻击力物理伤害。绿霸符：附近的友方英雄生命低于40%时回复12%最大生命（每人10秒一次）。
 （攻击间隔 1.33 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F204" s="2" t="inlineStr">
+      <c r="F205" s="2" t="inlineStr">
         <is>
           <t>疾行神龛：在脚下放下神龛（4秒），水花使周围敌人受到80 + 60% 法强魔法伤害并减速40%；神龛里的友方英雄移速+30%、攻速+25%。
 （冷却 7 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G204" s="2" t="inlineStr">
+      <c r="G205" s="2" t="inlineStr">
         <is>
           <t>蟹壳护盾：缩进壳里，获得120 + 60% 法强护盾（2秒）。护盾打光或到时间时蟹壳碎裂：周围敌人受到80 + 60% 法强魔法伤害、眩晕0.5秒并减速40%。
 （冷却 6 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H204" s="2" t="inlineStr">
+      <c r="H205" s="2" t="inlineStr">
         <is>
           <t>你挖得动吗？：钻入地下2.5秒：受到的伤害降低50%、免疫控制，持续回复250 + 80% 法强生命；然后钻出地面，周围敌人受到160 + 60% 攻击力物理伤害并被击飞1.5秒。
 （冷却 25 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I204" s="2" t="inlineStr"/>
-      <c r="J204" s="2" t="inlineStr">
+      <c r="I205" s="2" t="inlineStr"/>
+      <c r="J205" s="2" t="inlineStr">
         <is>
           <t>2.67</t>
         </is>
       </c>
-      <c r="K204" s="2" t="inlineStr"/>
-      <c r="L204" s="3" t="inlineStr">
+      <c r="K205" s="2" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scuttlecrab.md</t>
         </is>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="2" t="inlineStr">
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B205" s="2" t="inlineStr">
+      <c r="B206" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C205" s="2" t="inlineStr">
+      <c r="C206" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
+      <c r="D206" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E205" s="2" t="inlineStr">
+      <c r="E206" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F205" s="2" t="inlineStr">
+      <c r="F206" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G205" s="2" t="inlineStr">
+      <c r="G206" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H205" s="2" t="inlineStr">
+      <c r="H206" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I205" s="2" t="inlineStr"/>
-      <c r="J205" s="2" t="inlineStr">
+      <c r="I206" s="2" t="inlineStr"/>
+      <c r="J206" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K205" s="2" t="inlineStr"/>
-      <c r="L205" s="3" t="inlineStr">
+      <c r="K206" s="2" t="inlineStr"/>
+      <c r="L206" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L205"/>
+  <autoFilter ref="A1:L206"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13553,6 +13611,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L204" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L206" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Senna PPU 1.87 registered: league.dll 0.8.39 (hd.rs row), main 0.286.0; Illaoi's spirit, Viego's souls (her hd_ / lo_ tags; Neeko reads the same table) - league_viego_soul 0.2.47; preview_senna on the dense frames; hero page, gallery, tech notes, README
39 game px as her 1x sprite: no SIZES row, the face point (3, -36) stays (tfm2_ase face: PASS); her card unchanged
(bp_card_audit: fine). The idle and ban/pick reels are hero_reels' cuts of the new frames. Sylas's tables unchanged.
ui_sheets ok, every add-on's override check ok, league_main / league_viego_soul tests ok. Main merged first
(63f176930, #654; dll 0.8.38 / main 0.285.0 / viego 0.2.46 as installed). The user: 「赛娜没问题」.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.46）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.47）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -11033,7 +11033,7 @@
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="K166" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
tft_sentry: versions above #659 (main 0.288.0 / league.dll 0.8.41 / illaoi 0.2.44 needs main 0.288.0 / sylas 0.2.44 / viego_soul 0.2.48 / yuumi 0.2.3 / neeko 0.1.5 / tft 0.37.0); hero page (dev record), README (ADC 30, tft 33, 206), heroes.xlsx, previews
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/heroes.xlsx
+++ b/docs/heroes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="英雄" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$206</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英雄'!$A$1:$L$207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L206"/>
+  <dimension ref="A1:L207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>俄洛伊附加包（league_illaoi v0.2.43）
+          <t>俄洛伊附加包（league_illaoi v0.2.44）
 触手长在哪：按被动自己的冷却长（1 级 p_cd_1、18 级 p_cd_18，英雄联盟 20 – 10 秒，不再跟着普攻长），长在她附近最近的墙边（p_reach 内，没墙就在她身边 t_…
 触手抽谁：平时不动（英雄联盟）：严酷训诫打中的人（够得着的每条依次抽一下）、灵魂被扯出来的英雄和躯壳（每 t_per tick）；Q 并进被动：她打中敌人时够得着的触手抽一下（q_cd 一…
 灵魂分担伤害：只有她打他的每一下（普攻和技能，on_attack）多算 e_echo%，和英雄联盟打灵魂传到本体一样只算她的
@@ -5297,7 +5297,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.47）
+          <t>佛耶戈「君命已决」附加包（league_viego_soul v0.2.48）
 什么时候附身：读每个敌方英雄的死亡：他 3 秒内打过的英雄一死就算他的功劳，每个都算
 灵魂在哪：尸体那里留下灵魂 8 秒，35000 以内直接附身，90000 以内他冲过去附身（照英雄联盟要去拿那个灵魂）
 附身后的样子：整个身体变成被附身的那个英雄：站、跑、出招、挨打都是那个英雄的图（只在游戏 0.6.4 上，别的版本退回左边那样）
@@ -7020,7 +7020,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>妮蔻附加包（league_neeko v0.1.4）
+          <t>妮蔻附加包（league_neeko v0.1.5）
 天生幻魅：脱战 2 秒后整个身体画成最近的友方英雄（站、跑、出招、挨打都用他的图）；放技能、被控（击飞、晕眩、禁锢、嘲讽、恐惧、魅惑、强制位移）、假扮以来挨了她 35% 最大生命的伤害、或…</t>
         </is>
       </c>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>塞拉斯附加包（league_sylas v0.2.43）
+          <t>塞拉斯附加包（league_sylas v0.2.44）
 主包 league 保持纯数据。用户选了「做，含按类别偷大招+连招」，又要求「有连招要做连招」。主包的数据复制不了别的英雄的大招，也读不到当前生命，所以这两件事放在这个附加包里用原生代码做，外加连招： - 其人之道：偷到谁就放谁的大招（0.2.0，用户：「塞拉斯偷到谁就放谁的真大招」「只用管LOL的」）：偷到本包的英雄联盟英雄（src/stealable.…</t>
         </is>
       </c>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>悠米附加包（league_yuumi v0.2.1）
+          <t>悠米附加包（league_yuumi v0.2.3）
 附身多久：不限时，队友死了才跳下来；骑着时看局势换人：宿主闲着就跳去打架的队友，去救快死的队友，跟着中单 / 下路
 附身时能不能出招：能：Q、R、再给他一次旺盛精力（护盾 130 + 60% 法强 3 秒、攻速 +20%、移速 +10%），都从他头上放
 附身时谁能打到她：平时谁都打不到（一段一段地放逐）；出招的那一小段受到的伤害 -100%、免控
@@ -13117,295 +13117,353 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
+          <t>苍蓝哨戒</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Pebbles</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>tft_sentry</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>ADC</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>蓝核射出碎光弹，造成100% 攻击力物理伤害和45% 法强魔法伤害。青霸符：蔚蓝激光每引导1秒，大招冷却-1秒。
+（攻击间隔 1.2 秒 · 攻击距离 60000）</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>蔚蓝激光：对目标引导激光2.5秒（可以边飘边照），共造成460 + 250% 法强魔法伤害，每0.25秒魔抗-4（可叠加，持续2秒）。目标离开射程或自己被控时中断。
+（冷却 6 秒 · 施放距离 65000 · 施放：指定目标 · 敌人（不含防御塔））</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>裂石跃迁：两块石头猛地分开再合拢，周围敌人受到80 + 45% 法强魔法伤害并减速40%（1.5秒），自己向后闪开。
+（冷却 10 秒 · 施放距离 45000 · 施放：指定目标 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>棱镜扫射：两块石头张开，蓝核射出光柱扫过前方扇形，造成320 + 160% 法强魔法伤害，魔抗-25（3秒）。
+（冷却 35 秒 · 施放距离 70000 · 施放：地点 · 敌方英雄）</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_sentry.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
           <t>艾达丝</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
+      <c r="B203" s="2" t="inlineStr">
         <is>
           <t>Idas</t>
         </is>
       </c>
-      <c r="C202" s="2" t="inlineStr">
+      <c r="C203" s="2" t="inlineStr">
         <is>
           <t>tft_idas</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E202" s="2" t="inlineStr">
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>挥爪造成100% 攻击力物理伤害。护卫之誓：生命值低于50%时，她和最近的一名友军各获得她最大生命值18%的护盾（5秒），每30秒一次。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
+      <c r="F203" s="2" t="inlineStr">
         <is>
           <t>黄金龙息：向前喷出扇形金色龙息，造成110 + 70% 法强魔法伤害，护甲降低35%（4秒）。
 （冷却 5 秒 · 施放距离 35000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G202" s="2" t="inlineStr">
+      <c r="G203" s="2" t="inlineStr">
         <is>
           <t>龙威振翅：振翅一吼：附近的敌人眩晕0.75秒并减速50%（2秒）；她和附近友军获得50 + 30% 法强护盾（3秒）。
 （冷却 9 秒 · 施放距离 55000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H202" s="2" t="inlineStr">
+      <c r="H203" s="2" t="inlineStr">
         <is>
           <t>黄金龙鳞：双翼裹身2秒，受到的伤害降低60%；然后回复200 + 60% 法强生命值，附近友军获得150 + 50% 法强护盾（5秒），护盾在时攻速+30%。
 （冷却 25 秒 · 施放距离 70000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I202" s="2" t="inlineStr"/>
-      <c r="J202" s="2" t="inlineStr">
+      <c r="I203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
-      <c r="L202" s="3" t="inlineStr">
+      <c r="K203" s="2" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_idas.md</t>
         </is>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="2" t="inlineStr">
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
         <is>
           <t>洛里斯</t>
         </is>
       </c>
-      <c r="B203" s="2" t="inlineStr">
+      <c r="B204" s="2" t="inlineStr">
         <is>
           <t>Loris</t>
         </is>
       </c>
-      <c r="C203" s="2" t="inlineStr">
+      <c r="C204" s="2" t="inlineStr">
         <is>
           <t>tft_loris</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
+      <c r="D204" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E203" s="2" t="inlineStr">
+      <c r="E204" s="2" t="inlineStr">
         <is>
           <t>举盾猛砸，造成100% 攻击力物理伤害。神盾使：每条命第一次生命低于75%和25%时，各获得最大生命12%的护盾（4秒）。
 （攻击间隔 1.4 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F203" s="2" t="inlineStr">
+      <c r="F204" s="2" t="inlineStr">
         <is>
           <t>皮城争斗：获得70 + 50% 法强的护盾（4秒），举盾冲锋，撞到的敌人受到110 + 70% 法强魔法伤害并晕眩1.5秒。
 （冷却 7 秒 · 施放距离 42000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G203" s="2" t="inlineStr">
+      <c r="G204" s="2" t="inlineStr">
         <is>
           <t>盾卫：冲到附近生命比例最低的友方英雄身边，两人各获得70 + 45% 法强的护盾（4秒），期间替他承受30%的伤害。
 （冷却 10 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H203" s="2" t="inlineStr">
+      <c r="H204" s="2" t="inlineStr">
         <is>
           <t>钢铁防线：把巨盾砸进地里，周围的敌人受到220 + 80% 法强魔法伤害、被击飞1秒并嘲讽2秒；自己受到的伤害降低50%（4秒）。
 （冷却 50 秒 · 施放距离 30000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I203" s="2" t="inlineStr"/>
-      <c r="J203" s="2" t="inlineStr">
+      <c r="I204" s="2" t="inlineStr"/>
+      <c r="J204" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K203" s="2" t="inlineStr"/>
-      <c r="L203" s="3" t="inlineStr">
+      <c r="K204" s="2" t="inlineStr"/>
+      <c r="L204" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_loris.md</t>
         </is>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="2" t="inlineStr">
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
         <is>
           <t>小木灵</t>
         </is>
       </c>
-      <c r="B204" s="2" t="inlineStr">
+      <c r="B205" s="2" t="inlineStr">
         <is>
           <t>Meepsie</t>
         </is>
       </c>
-      <c r="C204" s="2" t="inlineStr">
+      <c r="C205" s="2" t="inlineStr">
         <is>
           <t>tft_meepsie</t>
         </is>
       </c>
-      <c r="D204" s="2" t="inlineStr">
+      <c r="D205" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E204" s="2" t="inlineStr">
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>挥出月岩重拳，造成100% 攻击力物理伤害。木灵驾驶员：每一拳额外造成15 + 25% 法强魔法伤害。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F204" s="2" t="inlineStr">
+      <c r="F205" s="2" t="inlineStr">
         <is>
           <t>月尘震地：一拳砸向前方地面，扇形范围内的敌人受到100 + 70% 法强魔法伤害并减速40%（2秒）。
 （冷却 6 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G204" s="2" t="inlineStr">
+      <c r="G205" s="2" t="inlineStr">
         <is>
           <t>治疗木灵：驾驶员一招手，4只小木灵飞向身边生命比例最低的队友（名额有剩时也治疗自己），每0.5秒回复20 + 10% 法强生命，持续3秒。
 （冷却 9 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H204" s="2" t="inlineStr">
+      <c r="H205" s="2" t="inlineStr">
         <is>
           <t>宇宙大爆炸：跳向附近敌方英雄最多的地方砸地，周围的敌人受到160 + 90% 法强魔法伤害，离中心每远一格少35%；离落点最近的3个敌方英雄被击飞1.25秒。
 （冷却 35 秒 · 施放距离 45000 · 施放：指定目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I204" s="2" t="inlineStr"/>
-      <c r="J204" s="2" t="inlineStr">
+      <c r="I205" s="2" t="inlineStr"/>
+      <c r="J205" s="2" t="inlineStr">
         <is>
           <t>2.88</t>
         </is>
       </c>
-      <c r="K204" s="2" t="inlineStr"/>
-      <c r="L204" s="3" t="inlineStr">
+      <c r="K205" s="2" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_meepsie.md</t>
         </is>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="2" t="inlineStr">
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
         <is>
           <t>迅捷蟹</t>
         </is>
       </c>
-      <c r="B205" s="2" t="inlineStr">
+      <c r="B206" s="2" t="inlineStr">
         <is>
           <t>Scuttle Crab</t>
         </is>
       </c>
-      <c r="C205" s="2" t="inlineStr">
+      <c r="C206" s="2" t="inlineStr">
         <is>
           <t>tft_scuttlecrab</t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
+      <c r="D206" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E205" s="2" t="inlineStr">
+      <c r="E206" s="2" t="inlineStr">
         <is>
           <t>跳一段螃蟹舞，踩中身边所有敌人，造成100% 攻击力物理伤害。绿霸符：附近的友方英雄生命低于40%时回复12%最大生命（每人10秒一次）。
 （攻击间隔 1.33 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F205" s="2" t="inlineStr">
+      <c r="F206" s="2" t="inlineStr">
         <is>
           <t>疾行神龛：在脚下放下神龛（4秒），水花使周围敌人受到80 + 60% 法强魔法伤害并减速40%；神龛里的友方英雄移速+30%、攻速+25%。
 （冷却 7 秒 · 施放距离 60000 · 施放：无目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G205" s="2" t="inlineStr">
+      <c r="G206" s="2" t="inlineStr">
         <is>
           <t>蟹壳护盾：缩进壳里，获得120 + 60% 法强护盾（2秒）。护盾打光或到时间时蟹壳碎裂：周围敌人受到80 + 60% 法强魔法伤害、眩晕0.5秒并减速40%。
 （冷却 6 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H205" s="2" t="inlineStr">
+      <c r="H206" s="2" t="inlineStr">
         <is>
           <t>你挖得动吗？：钻入地下2.5秒：受到的伤害降低50%、免疫控制，持续回复250 + 80% 法强生命；然后钻出地面，周围敌人受到160 + 60% 攻击力物理伤害并被击飞1.5秒。
 （冷却 25 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I205" s="2" t="inlineStr"/>
-      <c r="J205" s="2" t="inlineStr">
+      <c r="I206" s="2" t="inlineStr"/>
+      <c r="J206" s="2" t="inlineStr">
         <is>
           <t>2.67</t>
         </is>
       </c>
-      <c r="K205" s="2" t="inlineStr"/>
-      <c r="L205" s="3" t="inlineStr">
+      <c r="K206" s="2" t="inlineStr"/>
+      <c r="L206" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_scuttlecrab.md</t>
         </is>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="2" t="inlineStr">
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
         <is>
           <t>斯特卜</t>
         </is>
       </c>
-      <c r="B206" s="2" t="inlineStr">
+      <c r="B207" s="2" t="inlineStr">
         <is>
           <t>Steb</t>
         </is>
       </c>
-      <c r="C206" s="2" t="inlineStr">
+      <c r="C207" s="2" t="inlineStr">
         <is>
           <t>tft_steb</t>
         </is>
       </c>
-      <c r="D206" s="2" t="inlineStr">
+      <c r="D207" s="2" t="inlineStr">
         <is>
           <t>辅助</t>
         </is>
       </c>
-      <c r="E206" s="2" t="inlineStr">
+      <c r="E207" s="2" t="inlineStr">
         <is>
           <t>双警棍轮流打击，造成100% 攻击力物理伤害。战地医疗：自己受到治疗时，最近的2名友方英雄也回复该治疗量的25%。
 （攻击间隔 1.5 秒 · 攻击距离 25000）</t>
         </is>
       </c>
-      <c r="F206" s="2" t="inlineStr">
+      <c r="F207" s="2" t="inlineStr">
         <is>
           <t>战地医疗：给自己打一针，回复120 + 60% 法强生命，再重击目标造成170 + 120% 法强魔法伤害并眩晕0.75秒。
 （冷却 5.5 秒 · 施放距离 30000 · 施放：指定目标 · 敌人（不含防御塔））</t>
         </is>
       </c>
-      <c r="G206" s="2" t="inlineStr">
+      <c r="G207" s="2" t="inlineStr">
         <is>
           <t>通缉令：通缉附近生命最高的敌方英雄5秒：它受到的伤害提高25%；它在通缉中阵亡时，自己和附近友方攻速提高30%（5秒）。
 （冷却 10 秒 · 施放距离 60000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="H206" s="2" t="inlineStr">
+      <c r="H207" s="2" t="inlineStr">
         <is>
           <t>医疗背包：打开医疗背包：自己和周围友方英雄获得120 + 50% 法强的护盾（4秒），自己减伤30%；之后每0.5秒为周围友方回复25 + 12% 法强生命，共6次。
 （冷却 40 秒 · 施放距离 50000 · 施放：无目标 · 敌方英雄）</t>
         </is>
       </c>
-      <c r="I206" s="2" t="inlineStr"/>
-      <c r="J206" s="2" t="inlineStr">
+      <c r="I207" s="2" t="inlineStr"/>
+      <c r="J207" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="K206" s="2" t="inlineStr"/>
-      <c r="L206" s="3" t="inlineStr">
+      <c r="K207" s="2" t="inlineStr"/>
+      <c r="L207" s="3" t="inlineStr">
         <is>
           <t>https://github.com/BoDUD/TFM2-League-Heroes/blob/main/docs/heroes/tft_steb.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L206"/>
+  <autoFilter ref="A1:L207"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -13612,6 +13670,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L204" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L205" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L207" r:id="rId206"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>